<commit_message>
Implement USB port enablement feature with management API and UI updates
</commit_message>
<xml_diff>
--- a/documents/testing/ecube-qa-test-cases.xlsx
+++ b/documents/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I171"/>
+  <dimension ref="A1:I188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2080,12 +2080,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>§12.5 USB Hardware</t>
+          <t>§12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C59" s="3" t="n"/>
@@ -2099,27 +2099,27 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>TC-501</t>
+          <t>TC-431</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Hot-plug detection</t>
+          <t>List ports — admin</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Plug in a USB drive, wait 30 seconds</t>
+          <t>GET /admin/ports with admin token</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>GET /drives shows the new drive in AVAILABLE state (discovery auto-transitions EMPTY → AVAILABLE)</t>
+          <t>200, array of port objects with enabled field</t>
         </is>
       </c>
       <c r="F60" s="4" t="n"/>
@@ -2130,27 +2130,27 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>TC-502</t>
+          <t>TC-432</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>USB topology</t>
+          <t>List ports — manager</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/usb/topology</t>
+          <t>GET /admin/ports with manager token</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Shows real hub serial numbers, port numbers, connected devices</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F61" s="4" t="n"/>
@@ -2161,27 +2161,27 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>TC-503</t>
+          <t>TC-433</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Physical eject</t>
+          <t>List ports — processor denied</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Initialize drive → prepare-eject → physically remove</t>
+          <t>GET /admin/ports with processor token</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F62" s="4" t="n"/>
@@ -2192,27 +2192,27 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>TC-504</t>
+          <t>TC-434</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Re-plug same drive</t>
+          <t>List ports — unauthenticated</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Remove and re-insert the same drive</t>
+          <t>GET /admin/ports without token</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F63" s="4" t="n"/>
@@ -2223,27 +2223,27 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>TC-505</t>
+          <t>TC-435</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Multiple drives</t>
+          <t>Enable a port</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Plug in 2+ drives simultaneously</t>
+          <t>PATCH /admin/ports/{id} with {"enabled": true}</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>All drives appear in /drives; each can be initialized to different projects</t>
+          <t>200, port returned with enabled: true</t>
         </is>
       </c>
       <c r="F64" s="4" t="n"/>
@@ -2254,27 +2254,27 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>TC-506</t>
+          <t>TC-436</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Sync + unmount</t>
+          <t>Disable a port</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Initialize drive, create/start a job, then prepare-eject</t>
+          <t>PATCH /admin/ports/{id} with {"enabled": false}</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
+          <t>200, port returned with enabled: false</t>
         </is>
       </c>
       <c r="F65" s="4" t="n"/>
@@ -2283,48 +2283,60 @@
       <c r="I65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>§12.6 End-to-End Copy</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>12.6 End-to-End Copy</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="n"/>
-      <c r="I66" s="3" t="n"/>
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>TC-437</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>12.4.3 Port Enablement</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Enable port — manager</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/ports/{id} with manager token</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="n"/>
+      <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
+      <c r="I66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>TC-601</t>
+          <t>TC-438</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>12.6 End-to-End Copy</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Full E2E workflow</t>
+          <t>Enable port — processor denied</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Setup test files → add mount → discover drive → initialize → create job → start → poll → verify → manifest → eject → verify on another machine</t>
+          <t>PATCH /admin/ports/{id} with processor token</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>All steps succeed; checksums match; audit trail shows complete chain</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F67" s="4" t="n"/>
@@ -2333,44 +2345,60 @@
       <c r="I67" s="4" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>§12.7 Error Handling</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>12.7 Error Handling</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
-      <c r="G68" s="3" t="n"/>
-      <c r="H68" s="3" t="n"/>
-      <c r="I68" s="3" t="n"/>
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>TC-439</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>12.4.3 Port Enablement</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Enable non-existent port</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/ports/99999 with {"enabled": true}</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>404, NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n"/>
+      <c r="I68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>TC-701</t>
+          <t>TC-440</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/99999</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr"/>
+          <t>Ports default to disabled</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Discover a new port, then GET /admin/ports</t>
+        </is>
+      </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>New port has enabled: false</t>
         </is>
       </c>
       <c r="F69" s="4" t="n"/>
@@ -2381,23 +2409,27 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>TC-702</t>
+          <t>TC-441</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>DELETE /mounts/99999</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr"/>
+          <t>Drive on disabled port stays EMPTY</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Plug in drive on disabled port, run POST /drives/refresh</t>
+        </is>
+      </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>GET /drives shows drive in EMPTY state</t>
         </is>
       </c>
       <c r="F70" s="4" t="n"/>
@@ -2408,23 +2440,27 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>TC-703</t>
+          <t>TC-442</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Start an already-running job</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr"/>
+          <t>Drive on enabled port becomes AVAILABLE</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Enable port, run POST /drives/refresh</t>
+        </is>
+      </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>409, CONFLICT</t>
+          <t>GET /drives shows drive in AVAILABLE state</t>
         </is>
       </c>
       <c r="F71" s="4" t="n"/>
@@ -2435,23 +2471,27 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>TC-704</t>
+          <t>TC-443</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>All error responses</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr"/>
+          <t>Disable port — IN_USE drive unaffected</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Disable a port with an IN_USE drive, run POST /drives/refresh</t>
+        </is>
+      </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>JSON body includes code, message, and trace_id</t>
+          <t>Drive remains IN_USE (project isolation priority)</t>
         </is>
       </c>
       <c r="F72" s="4" t="n"/>
@@ -2462,23 +2502,27 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>TC-705</t>
+          <t>TC-444</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/999/format with {"filesystem_type": "ext4"}</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr"/>
+          <t>PORT_ENABLED audit log</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=PORT_ENABLED after enabling a port</t>
+        </is>
+      </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>Audit entry with port_id, system_path, hub_id</t>
         </is>
       </c>
       <c r="F73" s="4" t="n"/>
@@ -2489,23 +2533,27 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>TC-706</t>
+          <t>TC-445</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr"/>
+          <t>PORT_DISABLED audit log</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=PORT_DISABLED after disabling a port</t>
+        </is>
+      </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>422, validation error</t>
+          <t>Audit entry with port_id, system_path, hub_id</t>
         </is>
       </c>
       <c r="F74" s="4" t="n"/>
@@ -2514,75 +2562,79 @@
       <c r="I74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>TC-707</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>12.7 Error Handling</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/format with empty body</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr"/>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="n"/>
-      <c r="G75" s="4" t="n"/>
-      <c r="H75" s="4" t="n"/>
-      <c r="I75" s="4" t="n"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>§12.5 USB Hardware</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>12.5 USB Hardware</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="n"/>
+      <c r="D75" s="3" t="n"/>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="n"/>
+      <c r="G75" s="3" t="n"/>
+      <c r="H75" s="3" t="n"/>
+      <c r="I75" s="3" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>§12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="n"/>
-      <c r="D76" s="3" t="n"/>
-      <c r="E76" s="3" t="n"/>
-      <c r="F76" s="3" t="n"/>
-      <c r="G76" s="3" t="n"/>
-      <c r="H76" s="3" t="n"/>
-      <c r="I76" s="3" t="n"/>
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>TC-501</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>12.5 USB Hardware</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Hot-plug detection</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Plug in a USB drive, wait 30 seconds</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>GET /drives shows the new drive (in EMPTY state if port is disabled, or AVAILABLE if port is enabled)</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>TC-801</t>
+          <t>TC-502</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>List users (empty)</t>
+          <t>USB topology</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>GET /users with admin token (no roles assigned yet)</t>
+          <t>GET /introspection/usb/topology</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>200, {"users": []}</t>
+          <t>Shows real hub serial numbers, port numbers, connected devices</t>
         </is>
       </c>
       <c r="F77" s="4" t="n"/>
@@ -2593,27 +2645,27 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>TC-802</t>
+          <t>TC-503</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Assign roles</t>
+          <t>Physical eject</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["processor", "auditor"]}</t>
+          <t>Initialize drive → prepare-eject → physically remove</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>200, returns username and sorted roles</t>
+          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
         </is>
       </c>
       <c r="F78" s="4" t="n"/>
@@ -2624,27 +2676,27 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>TC-803</t>
+          <t>TC-504</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Get roles</t>
+          <t>Re-plug same drive</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>GET /users/qa-processor/roles after assignment</t>
+          <t>Remove and re-insert the same drive</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
+          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
         </is>
       </c>
       <c r="F79" s="4" t="n"/>
@@ -2655,27 +2707,27 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>TC-804</t>
+          <t>TC-505</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>List users after assignment</t>
+          <t>Multiple drives</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>GET /users after assigning roles</t>
+          <t>Plug in 2+ drives simultaneously</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>200, user appears in list with correct roles</t>
+          <t>All drives appear in /drives; each can be initialized to different projects</t>
         </is>
       </c>
       <c r="F80" s="4" t="n"/>
@@ -2686,27 +2738,27 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>TC-805</t>
+          <t>TC-506</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Replace roles</t>
+          <t>Sync + unmount</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["manager"]}</t>
+          <t>Initialize drive, create/start a job, then prepare-eject</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>200, only ["manager"] returned; old roles removed</t>
+          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
         </is>
       </c>
       <c r="F81" s="4" t="n"/>
@@ -2717,27 +2769,27 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>TC-806</t>
+          <t>TC-507</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Deduplicate roles</t>
+          <t>Disabled port blocks AVAILABLE</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
+          <t>Disable a port, plug in a drive to that port, run discovery</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>200, deduplicated to ["admin", "processor"]</t>
+          <t>Drive appears in EMPTY state; enable port + refresh → drive transitions to AVAILABLE</t>
         </is>
       </c>
       <c r="F82" s="4" t="n"/>
@@ -2746,60 +2798,48 @@
       <c r="I82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>TC-807</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Invalid role name</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>422, error message mentions superuser</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="n"/>
-      <c r="G83" s="4" t="n"/>
-      <c r="H83" s="4" t="n"/>
-      <c r="I83" s="4" t="n"/>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>§12.6 End-to-End Copy</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>12.6 End-to-End Copy</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="n"/>
+      <c r="D83" s="3" t="n"/>
+      <c r="E83" s="3" t="n"/>
+      <c r="F83" s="3" t="n"/>
+      <c r="G83" s="3" t="n"/>
+      <c r="H83" s="3" t="n"/>
+      <c r="I83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>TC-808</t>
+          <t>TC-601</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.6 End-to-End Copy</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Empty role list</t>
+          <t>Full E2E workflow</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
+          <t>Setup test files → add mount → discover drive → initialize → create job → start → poll → verify → manifest → eject → verify on another machine</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>422, at least one role required</t>
+          <t>All steps succeed; checksums match; audit trail shows complete chain</t>
         </is>
       </c>
       <c r="F84" s="4" t="n"/>
@@ -2808,60 +2848,44 @@
       <c r="I84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>TC-809</t>
-        </is>
-      </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Remove roles</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>DELETE /users/qa-processor/roles</t>
-        </is>
-      </c>
-      <c r="E85" s="4" t="inlineStr">
-        <is>
-          <t>200, {"username": "qa-processor", "roles": []}</t>
-        </is>
-      </c>
-      <c r="F85" s="4" t="n"/>
-      <c r="G85" s="4" t="n"/>
-      <c r="H85" s="4" t="n"/>
-      <c r="I85" s="4" t="n"/>
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>§12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="n"/>
+      <c r="D85" s="3" t="n"/>
+      <c r="E85" s="3" t="n"/>
+      <c r="F85" s="3" t="n"/>
+      <c r="G85" s="3" t="n"/>
+      <c r="H85" s="3" t="n"/>
+      <c r="I85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>TC-810</t>
+          <t>TC-701</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Get roles after removal</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>GET /users/qa-processor/roles after DELETE</t>
-        </is>
-      </c>
+          <t>GET /jobs/99999</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr"/>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>200, {"roles": []}</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F86" s="4" t="n"/>
@@ -2872,27 +2896,23 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>TC-811</t>
+          <t>TC-702</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Get roles for unknown user</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>GET /users/nonexistent/roles</t>
-        </is>
-      </c>
+          <t>DELETE /mounts/99999</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr"/>
       <c r="E87" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "nonexistent", "roles": []}</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F87" s="4" t="n"/>
@@ -2903,27 +2923,23 @@
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>TC-812</t>
+          <t>TC-703</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot list users</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>GET /users with processor token</t>
-        </is>
-      </c>
+          <t>Start an already-running job</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr"/>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>409, CONFLICT</t>
         </is>
       </c>
       <c r="F88" s="4" t="n"/>
@@ -2934,27 +2950,23 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>TC-813</t>
+          <t>TC-704</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot set roles</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>PUT /users/x/roles with processor token</t>
-        </is>
-      </c>
+          <t>All error responses</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr"/>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>JSON body includes code, message, and trace_id</t>
         </is>
       </c>
       <c r="F89" s="4" t="n"/>
@@ -2965,27 +2977,23 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>TC-814</t>
+          <t>TC-705</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot delete roles</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>DELETE /users/x/roles with processor token</t>
-        </is>
-      </c>
+          <t>POST /drives/999/format with {"filesystem_type": "ext4"}</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr"/>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F90" s="4" t="n"/>
@@ -2996,27 +3004,23 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>TC-815</t>
+          <t>TC-706</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated access</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>GET /users without Authorization header</t>
-        </is>
-      </c>
+          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr"/>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>422, validation error</t>
         </is>
       </c>
       <c r="F91" s="4" t="n"/>
@@ -3027,27 +3031,23 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>TC-816</t>
+          <t>TC-707</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>ROLE_ASSIGNED audit log</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>GET /audit?action=ROLE_ASSIGNED after assigning roles</t>
-        </is>
-      </c>
+          <t>POST /drives/{id}/format with empty body</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr"/>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor, target user, and roles</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F92" s="4" t="n"/>
@@ -3056,40 +3056,28 @@
       <c r="I92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="inlineStr">
-        <is>
-          <t>TC-817</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>§12.8 User Role Mgmt</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>ROLE_REMOVED audit log</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>GET /audit?action=ROLE_REMOVED after removing roles</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>Audit entry with actor and target user</t>
-        </is>
-      </c>
-      <c r="F93" s="4" t="n"/>
-      <c r="G93" s="4" t="n"/>
-      <c r="H93" s="4" t="n"/>
-      <c r="I93" s="4" t="n"/>
+      <c r="C93" s="3" t="n"/>
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="3" t="n"/>
+      <c r="F93" s="3" t="n"/>
+      <c r="G93" s="3" t="n"/>
+      <c r="H93" s="3" t="n"/>
+      <c r="I93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>TC-818</t>
+          <t>TC-801</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
@@ -3099,17 +3087,17 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>DB roles override groups</t>
+          <t>List users (empty)</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
+          <t>GET /users with admin token (no roles assigned yet)</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
+          <t>200, {"users": []}</t>
         </is>
       </c>
       <c r="F94" s="4" t="n"/>
@@ -3120,7 +3108,7 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>TC-819</t>
+          <t>TC-802</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
@@ -3130,17 +3118,17 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Fallback to group roles</t>
+          <t>Assign roles</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["processor", "auditor"]}</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
         <is>
-          <t>JWT roles falls back to OS group mapping (["processor"])</t>
+          <t>200, returns username and sorted roles</t>
         </is>
       </c>
       <c r="F95" s="4" t="n"/>
@@ -3149,48 +3137,60 @@
       <c r="I95" s="4" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>§12.9 OS User &amp; Group Mgmt</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
-        </is>
-      </c>
-      <c r="C96" s="3" t="n"/>
-      <c r="D96" s="3" t="n"/>
-      <c r="E96" s="3" t="n"/>
-      <c r="F96" s="3" t="n"/>
-      <c r="G96" s="3" t="n"/>
-      <c r="H96" s="3" t="n"/>
-      <c r="I96" s="3" t="n"/>
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>TC-803</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>12.8 User Role Mgmt</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Get roles</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>GET /users/qa-processor/roles after assignment</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>TC-901</t>
+          <t>TC-804</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Create group</t>
+          <t>List users after assignment</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
+          <t>GET /users after assigning roles</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>201, returns name, gid, members</t>
+          <t>200, user appears in list with correct roles</t>
         </is>
       </c>
       <c r="F97" s="4" t="n"/>
@@ -3201,27 +3201,27 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>TC-902</t>
+          <t>TC-805</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Create group without prefix</t>
+          <t>Replace roles</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-groups with {"name": "testers"}</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["manager"]}</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>422, group name must start with ecube-</t>
+          <t>200, only ["manager"] returned; old roles removed</t>
         </is>
       </c>
       <c r="F98" s="4" t="n"/>
@@ -3232,27 +3232,27 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>TC-903</t>
+          <t>TC-806</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>List groups</t>
+          <t>Deduplicate roles</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-groups</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>200, only ecube-* groups listed</t>
+          <t>200, deduplicated to ["admin", "processor"]</t>
         </is>
       </c>
       <c r="F99" s="4" t="n"/>
@@ -3263,27 +3263,27 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>TC-904</t>
+          <t>TC-807</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Delete group</t>
+          <t>Invalid role name</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-groups/ecube-testers</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>422, error message mentions superuser</t>
         </is>
       </c>
       <c r="F100" s="4" t="n"/>
@@ -3294,27 +3294,27 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>TC-905</t>
+          <t>TC-808</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Delete group without prefix</t>
+          <t>Empty role list</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-groups/somegroup</t>
+          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>422, group name must start with ecube-</t>
+          <t>422, at least one role required</t>
         </is>
       </c>
       <c r="F101" s="4" t="n"/>
@@ -3325,27 +3325,27 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>TC-906</t>
+          <t>TC-809</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Create user</t>
+          <t>Remove roles</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with username, password, groups, roles</t>
+          <t>DELETE /users/qa-processor/roles</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>201, returns username, uid, gid, home, shell, groups</t>
+          <t>200, {"username": "qa-processor", "roles": []}</t>
         </is>
       </c>
       <c r="F102" s="4" t="n"/>
@@ -3356,27 +3356,27 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>TC-907</t>
+          <t>TC-810</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Create user — duplicate</t>
+          <t>Get roles after removal</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with existing username</t>
+          <t>GET /users/qa-processor/roles after DELETE</t>
         </is>
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200, {"roles": []}</t>
         </is>
       </c>
       <c r="F103" s="4" t="n"/>
@@ -3387,27 +3387,27 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>TC-908</t>
+          <t>TC-811</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Create user — reserved name</t>
+          <t>Get roles for unknown user</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"username": "root", ...}</t>
+          <t>GET /users/nonexistent/roles</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>422, reserved username</t>
+          <t>200, {"username": "nonexistent", "roles": []}</t>
         </is>
       </c>
       <c r="F104" s="4" t="n"/>
@@ -3418,27 +3418,27 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>TC-909</t>
+          <t>TC-812</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Create user — empty password</t>
+          <t>Processor cannot list users</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"password": "", ...}</t>
+          <t>GET /users with processor token</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F105" s="4" t="n"/>
@@ -3449,27 +3449,27 @@
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>TC-910</t>
+          <t>TC-813</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with newline</t>
+          <t>Processor cannot set roles</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing \n</t>
+          <t>PUT /users/x/roles with processor token</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F106" s="4" t="n"/>
@@ -3480,27 +3480,27 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>TC-911</t>
+          <t>TC-814</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with colon</t>
+          <t>Processor cannot delete roles</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing :</t>
+          <t>DELETE /users/x/roles with processor token</t>
         </is>
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F107" s="4" t="n"/>
@@ -3511,27 +3511,27 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>TC-912</t>
+          <t>TC-815</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Create user — invalid group</t>
+          <t>Unauthenticated access</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with non-existent group in groups list</t>
+          <t>GET /users without Authorization header</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>422, group does not exist</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F108" s="4" t="n"/>
@@ -3542,27 +3542,27 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>TC-913</t>
+          <t>TC-816</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Create user — no ecube-* group</t>
+          <t>ROLE_ASSIGNED audit log</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
+          <t>GET /audit?action=ROLE_ASSIGNED after assigning roles</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>Audit entry with actor, target user, and roles</t>
         </is>
       </c>
       <c r="F109" s="4" t="n"/>
@@ -3573,27 +3573,27 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>TC-914</t>
+          <t>TC-817</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>List users</t>
+          <t>ROLE_REMOVED audit log</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users</t>
+          <t>GET /audit?action=ROLE_REMOVED after removing roles</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>200, only users in ecube-* groups listed</t>
+          <t>Audit entry with actor and target user</t>
         </is>
       </c>
       <c r="F110" s="4" t="n"/>
@@ -3604,27 +3604,27 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>TC-915</t>
+          <t>TC-818</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Reset password</t>
+          <t>DB roles override groups</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
         </is>
       </c>
       <c r="F111" s="4" t="n"/>
@@ -3635,27 +3635,27 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>TC-916</t>
+          <t>TC-819</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Reset password — non-ECUBE user</t>
+          <t>Fallback to group roles</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/postgres/password</t>
+          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>JWT roles falls back to OS group mapping (["processor"])</t>
         </is>
       </c>
       <c r="F112" s="4" t="n"/>
@@ -3664,40 +3664,28 @@
       <c r="I112" s="4" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>TC-917</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>§12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>Replace groups</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>200, updated group list; non-ecube-* groups preserved</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="n"/>
-      <c r="G113" s="4" t="n"/>
-      <c r="H113" s="4" t="n"/>
-      <c r="I113" s="4" t="n"/>
+      <c r="C113" s="3" t="n"/>
+      <c r="D113" s="3" t="n"/>
+      <c r="E113" s="3" t="n"/>
+      <c r="F113" s="3" t="n"/>
+      <c r="G113" s="3" t="n"/>
+      <c r="H113" s="3" t="n"/>
+      <c r="I113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>TC-918</t>
+          <t>TC-901</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
@@ -3707,17 +3695,17 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — empty list</t>
+          <t>Create group</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
+          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>201, returns name, gid, members</t>
         </is>
       </c>
       <c r="F114" s="4" t="n"/>
@@ -3728,7 +3716,7 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>TC-919</t>
+          <t>TC-902</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
@@ -3738,17 +3726,17 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — non-ecube name</t>
+          <t>Create group without prefix</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
+          <t>POST /admin/os-groups with {"name": "testers"}</t>
         </is>
       </c>
       <c r="E115" s="4" t="inlineStr">
         <is>
-          <t>422, group does not start with ecube-</t>
+          <t>422, group name must start with ecube-</t>
         </is>
       </c>
       <c r="F115" s="4" t="n"/>
@@ -3759,7 +3747,7 @@
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>TC-920</t>
+          <t>TC-903</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -3769,17 +3757,17 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Append groups</t>
+          <t>List groups</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+          <t>GET /admin/os-groups</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
+          <t>200, only ecube-* groups listed</t>
         </is>
       </c>
       <c r="F116" s="4" t="n"/>
@@ -3790,7 +3778,7 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>TC-921</t>
+          <t>TC-904</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -3800,17 +3788,17 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Modify groups — non-ECUBE user</t>
+          <t>Delete group</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/www-data/groups</t>
+          <t>DELETE /admin/os-groups/ecube-testers</t>
         </is>
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F117" s="4" t="n"/>
@@ -3821,7 +3809,7 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>TC-922</t>
+          <t>TC-905</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -3831,17 +3819,17 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Delete user</t>
+          <t>Delete group without prefix</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/{username}</t>
+          <t>DELETE /admin/os-groups/somegroup</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>200, user and DB roles removed</t>
+          <t>422, group name must start with ecube-</t>
         </is>
       </c>
       <c r="F118" s="4" t="n"/>
@@ -3852,7 +3840,7 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>TC-923</t>
+          <t>TC-906</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -3862,17 +3850,17 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Delete user — non-ECUBE user</t>
+          <t>Create user</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/daemon</t>
+          <t>POST /admin/os-users with username, password, groups, roles</t>
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>201, returns username, uid, gid, home, shell, groups</t>
         </is>
       </c>
       <c r="F119" s="4" t="n"/>
@@ -3883,7 +3871,7 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>TC-924</t>
+          <t>TC-907</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -3893,17 +3881,17 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Delete user — not found</t>
+          <t>Create user — duplicate</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/nonexistent</t>
+          <t>POST /admin/os-users with existing username</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F120" s="4" t="n"/>
@@ -3914,7 +3902,7 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>TC-925</t>
+          <t>TC-908</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -3924,17 +3912,17 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot access OS endpoints</t>
+          <t>Create user — reserved name</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users with processor token</t>
+          <t>POST /admin/os-users with {"username": "root", ...}</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>422, reserved username</t>
         </is>
       </c>
       <c r="F121" s="4" t="n"/>
@@ -3945,7 +3933,7 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>TC-926</t>
+          <t>TC-909</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -3955,17 +3943,17 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Non-local mode returns 404</t>
+          <t>Create user — empty password</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+          <t>POST /admin/os-users with {"password": "", ...}</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>404, Not Found</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F122" s="4" t="n"/>
@@ -3976,7 +3964,7 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>TC-927</t>
+          <t>TC-910</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
@@ -3986,17 +3974,17 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_CREATED audit log</t>
+          <t>Create user — password with newline</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+          <t>POST /admin/os-users with password containing \n</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F123" s="4" t="n"/>
@@ -4007,7 +3995,7 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>TC-928</t>
+          <t>TC-911</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -4017,17 +4005,17 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_DELETED audit log</t>
+          <t>Create user — password with colon</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+          <t>POST /admin/os-users with password containing :</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F124" s="4" t="n"/>
@@ -4038,7 +4026,7 @@
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>TC-929</t>
+          <t>TC-912</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -4048,17 +4036,17 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>OS_PASSWORD_RESET audit log</t>
+          <t>Create user — invalid group</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+          <t>POST /admin/os-users with non-existent group in groups list</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>Audit entry (no password in details)</t>
+          <t>422, group does not exist</t>
         </is>
       </c>
       <c r="F125" s="4" t="n"/>
@@ -4069,7 +4057,7 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>TC-930</t>
+          <t>TC-913</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -4079,17 +4067,17 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_CREATED audit log</t>
+          <t>Create user — no ecube-* group</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F126" s="4" t="n"/>
@@ -4100,7 +4088,7 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>TC-931</t>
+          <t>TC-914</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -4110,17 +4098,17 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_DELETED audit log</t>
+          <t>List users</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+          <t>GET /admin/os-users</t>
         </is>
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>200, only users in ecube-* groups listed</t>
         </is>
       </c>
       <c r="F127" s="4" t="n"/>
@@ -4129,48 +4117,60 @@
       <c r="I127" s="4" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>§12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C128" s="3" t="n"/>
-      <c r="D128" s="3" t="n"/>
-      <c r="E128" s="3" t="n"/>
-      <c r="F128" s="3" t="n"/>
-      <c r="G128" s="3" t="n"/>
-      <c r="H128" s="3" t="n"/>
-      <c r="I128" s="3" t="n"/>
+      <c r="A128" s="4" t="inlineStr">
+        <is>
+          <t>TC-915</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>Reset password</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="n"/>
+      <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n"/>
+      <c r="I128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>TC-1001</t>
+          <t>TC-916</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>Reset password — non-ECUBE user</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>PUT /admin/os-users/postgres/password</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F129" s="4" t="n"/>
@@ -4181,27 +4181,27 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>TC-1002</t>
+          <t>TC-917</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>Replace groups</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with valid username and password</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>200, updated group list; non-ecube-* groups preserved</t>
         </is>
       </c>
       <c r="F130" s="4" t="n"/>
@@ -4212,27 +4212,27 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-918</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Replace groups — empty list</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
         </is>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F131" s="4" t="n"/>
@@ -4243,27 +4243,27 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-919</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>Replace groups — non-ecube name</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>422, group does not start with ecube-</t>
         </is>
       </c>
       <c r="F132" s="4" t="n"/>
@@ -4274,27 +4274,27 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-920</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Append groups</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, updated group list</t>
         </is>
       </c>
       <c r="F133" s="4" t="n"/>
@@ -4305,27 +4305,27 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-921</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F134" s="4" t="n"/>
@@ -4336,27 +4336,27 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-922</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Delete user</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>200, user and DB roles removed</t>
         </is>
       </c>
       <c r="F135" s="4" t="n"/>
@@ -4367,27 +4367,27 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-923</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F136" s="4" t="n"/>
@@ -4398,27 +4398,27 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-924</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Delete user — not found</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>DELETE /admin/os-users/nonexistent</t>
         </is>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>404</t>
         </is>
       </c>
       <c r="F137" s="4" t="n"/>
@@ -4427,48 +4427,60 @@
       <c r="I137" s="4" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C138" s="3" t="n"/>
-      <c r="D138" s="3" t="n"/>
-      <c r="E138" s="3" t="n"/>
-      <c r="F138" s="3" t="n"/>
-      <c r="G138" s="3" t="n"/>
-      <c r="H138" s="3" t="n"/>
-      <c r="I138" s="3" t="n"/>
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>TC-925</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>Processor cannot access OS endpoints</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>GET /admin/os-users with processor token</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>403, FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="n"/>
+      <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n"/>
+      <c r="I138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-926</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Test connection — success</t>
+          <t>Non-local mode returns 404</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "ok", "server_version": "..."}</t>
+          <t>404, Not Found</t>
         </is>
       </c>
       <c r="F139" s="4" t="n"/>
@@ -4479,27 +4491,27 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-927</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Test connection — bad host</t>
+          <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with unreachable host</t>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F140" s="4" t="n"/>
@@ -4510,27 +4522,27 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-928</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Test connection — SSRF host</t>
+          <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>422, invalid host</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F141" s="4" t="n"/>
@@ -4541,27 +4553,27 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-929</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>Test connection — port out of range</t>
+          <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "port": 99999</t>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Audit entry (no password in details)</t>
         </is>
       </c>
       <c r="F142" s="4" t="n"/>
@@ -4572,27 +4584,27 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-930</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>Provision — success</t>
+          <t>OS_GROUP_CREATED audit log</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials</t>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F143" s="4" t="n"/>
@@ -4603,27 +4615,27 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-931</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>Provision — bad admin credentials</t>
+          <t>OS_GROUP_DELETED audit log</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with wrong admin password</t>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F144" s="4" t="n"/>
@@ -4632,60 +4644,48 @@
       <c r="I144" s="4" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="4" t="inlineStr">
-        <is>
-          <t>TC-1107</t>
-        </is>
-      </c>
-      <c r="B145" s="4" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C145" s="4" t="inlineStr">
-        <is>
-          <t>Provision — invalid database name</t>
-        </is>
-      </c>
-      <c r="D145" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
-        </is>
-      </c>
-      <c r="E145" s="4" t="inlineStr">
-        <is>
-          <t>422, invalid identifier</t>
-        </is>
-      </c>
-      <c r="F145" s="4" t="n"/>
-      <c r="G145" s="4" t="n"/>
-      <c r="H145" s="4" t="n"/>
-      <c r="I145" s="4" t="n"/>
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>§12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="n"/>
+      <c r="D145" s="3" t="n"/>
+      <c r="E145" s="3" t="n"/>
+      <c r="F145" s="3" t="n"/>
+      <c r="G145" s="3" t="n"/>
+      <c r="H145" s="3" t="n"/>
+      <c r="I145" s="3" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Status — connected</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with admin token</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>200, connected: true, migration info</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F146" s="4" t="n"/>
@@ -4696,27 +4696,27 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
         <is>
-          <t>Status — requires auth</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status without token</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E147" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F147" s="4" t="n"/>
@@ -4727,27 +4727,27 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Status — requires admin</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with processor token</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F148" s="4" t="n"/>
@@ -4758,27 +4758,27 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Settings update — success</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with valid partial update</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "updated", ...}</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>
@@ -4789,27 +4789,27 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Settings update — bad connection</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with unreachable host</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>400, connection test failed</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F150" s="4" t="n"/>
@@ -4820,27 +4820,27 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Settings update — empty body</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with {}</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>422, at least one field required</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F151" s="4" t="n"/>
@@ -4851,27 +4851,27 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Settings update — requires admin</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with processor token</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F152" s="4" t="n"/>
@@ -4882,27 +4882,27 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1008</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — test-connection</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F153" s="4" t="n"/>
@@ -4913,27 +4913,27 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>TC-1116</t>
+          <t>TC-1009</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — provision</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision without token (after admin exists)</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F154" s="4" t="n"/>
@@ -4942,40 +4942,28 @@
       <c r="I154" s="4" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="4" t="inlineStr">
-        <is>
-          <t>TC-1117</t>
-        </is>
-      </c>
-      <c r="B155" s="4" t="inlineStr">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C155" s="4" t="inlineStr">
-        <is>
-          <t>Password redaction</t>
-        </is>
-      </c>
-      <c r="D155" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/database/provision and check response</t>
-        </is>
-      </c>
-      <c r="E155" s="4" t="inlineStr">
-        <is>
-          <t>No password in response body</t>
-        </is>
-      </c>
-      <c r="F155" s="4" t="n"/>
-      <c r="G155" s="4" t="n"/>
-      <c r="H155" s="4" t="n"/>
-      <c r="I155" s="4" t="n"/>
+      <c r="C155" s="3" t="n"/>
+      <c r="D155" s="3" t="n"/>
+      <c r="E155" s="3" t="n"/>
+      <c r="F155" s="3" t="n"/>
+      <c r="G155" s="3" t="n"/>
+      <c r="H155" s="3" t="n"/>
+      <c r="I155" s="3" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>TC-1118</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
@@ -4985,17 +4973,17 @@
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Re-provision blocked</t>
+          <t>Test connection — success</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>409, already provisioned</t>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
       <c r="F156" s="4" t="n"/>
@@ -5006,7 +4994,7 @@
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>TC-1119</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B157" s="4" t="inlineStr">
@@ -5016,17 +5004,17 @@
       </c>
       <c r="C157" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision (admin)</t>
+          <t>Test connection — bad host</t>
         </is>
       </c>
       <c r="D157" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+          <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
       <c r="E157" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F157" s="4" t="n"/>
@@ -5037,7 +5025,7 @@
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>TC-1120</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -5047,17 +5035,17 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Force rejected unauthenticated</t>
+          <t>Test connection — SSRF host</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>403, force requires admin</t>
+          <t>422, invalid host</t>
         </is>
       </c>
       <c r="F158" s="4" t="n"/>
@@ -5068,7 +5056,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>TC-1121</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -5078,17 +5066,17 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Test connection — port out of range</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F159" s="4" t="n"/>
@@ -5099,7 +5087,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>TC-1122</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -5109,17 +5097,17 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Provision — success</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F160" s="4" t="n"/>
@@ -5130,7 +5118,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>TC-1123</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -5140,17 +5128,17 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — provision state unknown</t>
+          <t>Provision — bad admin credentials</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+          <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F161" s="4" t="n"/>
@@ -5161,7 +5149,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>TC-1124</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -5171,17 +5159,17 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Force bypasses state check</t>
+          <t>Provision — invalid database name</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>Proceeds to provisioning (no 503 from state check)</t>
+          <t>422, invalid identifier</t>
         </is>
       </c>
       <c r="F162" s="4" t="n"/>
@@ -5192,7 +5180,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>TC-1125</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -5202,17 +5190,17 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Unmigrated DB treated as initial setup</t>
+          <t>Status — connected</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>200, request allowed (not 503)</t>
+          <t>200, connected: true, migration info</t>
         </is>
       </c>
       <c r="F163" s="4" t="n"/>
@@ -5223,7 +5211,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>TC-1126</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -5233,17 +5221,17 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Fresh install — DB/role missing</t>
+          <t>Status — requires auth</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+          <t>GET /setup/database/status without token</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>200, provisioning proceeds (not 503)</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F164" s="4" t="n"/>
@@ -5254,7 +5242,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>TC-1127</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -5264,17 +5252,17 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — OperationalError on reachable DB</t>
+          <t>Status — requires admin</t>
         </is>
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F165" s="4" t="n"/>
@@ -5285,7 +5273,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>TC-1128</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -5295,17 +5283,17 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — unexpected error</t>
+          <t>Settings update — success</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+          <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
       <c r="F166" s="4" t="n"/>
@@ -5316,7 +5304,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>TC-1129</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -5326,17 +5314,17 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Provision — migration failure</t>
+          <t>Settings update — bad connection</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+          <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+          <t>400, connection test failed</t>
         </is>
       </c>
       <c r="F167" s="4" t="n"/>
@@ -5347,7 +5335,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>TC-1130</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -5357,17 +5345,17 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Provision — .env write failure</t>
+          <t>Settings update — empty body</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+          <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>500, "failed to persist" message; engine not swapped</t>
+          <t>422, at least one field required</t>
         </is>
       </c>
       <c r="F168" s="4" t="n"/>
@@ -5378,7 +5366,7 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>TC-1131</t>
+          <t>TC-1114</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
@@ -5388,17 +5376,17 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Provision — engine reinit failure</t>
+          <t>Settings update — requires admin</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+          <t>PUT /setup/database/settings with processor token</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>500, "engine could not be switched" message; .env already written</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F169" s="4" t="n"/>
@@ -5406,14 +5394,541 @@
       <c r="H169" s="4" t="n"/>
       <c r="I169" s="4" t="n"/>
     </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>TC-1115</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>Auth after setup — test-connection</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="n"/>
+      <c r="G170" s="4" t="n"/>
+      <c r="H170" s="4" t="n"/>
+      <c r="I170" s="4" t="n"/>
+    </row>
     <row r="171">
-      <c r="A171" s="5" t="inlineStr">
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>TC-1116</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t>Auth after setup — provision</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E171" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F171" s="4" t="n"/>
+      <c r="G171" s="4" t="n"/>
+      <c r="H171" s="4" t="n"/>
+      <c r="I171" s="4" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>TC-1117</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C172" s="4" t="inlineStr">
+        <is>
+          <t>Password redaction</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision and check response</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr">
+        <is>
+          <t>No password in response body</t>
+        </is>
+      </c>
+      <c r="F172" s="4" t="n"/>
+      <c r="G172" s="4" t="n"/>
+      <c r="H172" s="4" t="n"/>
+      <c r="I172" s="4" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="4" t="inlineStr">
+        <is>
+          <t>TC-1118</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t>Re-provision blocked</t>
+        </is>
+      </c>
+      <c r="D173" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+        </is>
+      </c>
+      <c r="E173" s="4" t="inlineStr">
+        <is>
+          <t>409, already provisioned</t>
+        </is>
+      </c>
+      <c r="F173" s="4" t="n"/>
+      <c r="G173" s="4" t="n"/>
+      <c r="H173" s="4" t="n"/>
+      <c r="I173" s="4" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>TC-1119</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t>Force re-provision (admin)</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr">
+        <is>
+          <t>200, returns database, user, migrations_applied</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="n"/>
+      <c r="G174" s="4" t="n"/>
+      <c r="H174" s="4" t="n"/>
+      <c r="I174" s="4" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="4" t="inlineStr">
+        <is>
+          <t>TC-1120</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t>Force rejected unauthenticated</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="inlineStr">
+        <is>
+          <t>403, force requires admin</t>
+        </is>
+      </c>
+      <c r="F175" s="4" t="n"/>
+      <c r="G175" s="4" t="n"/>
+      <c r="H175" s="4" t="n"/>
+      <c r="I175" s="4" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t>TC-1121</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, no JWT</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="inlineStr">
+        <is>
+          <t>503, database unavailable message</t>
+        </is>
+      </c>
+      <c r="F176" s="4" t="n"/>
+      <c r="G176" s="4" t="n"/>
+      <c r="H176" s="4" t="n"/>
+      <c r="I176" s="4" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>TC-1122</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="inlineStr">
+        <is>
+          <t>Request proceeds (not blocked by 503)</t>
+        </is>
+      </c>
+      <c r="F177" s="4" t="n"/>
+      <c r="G177" s="4" t="n"/>
+      <c r="H177" s="4" t="n"/>
+      <c r="I177" s="4" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="4" t="inlineStr">
+        <is>
+          <t>TC-1123</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — provision state unknown</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="inlineStr">
+        <is>
+          <t>503, cannot determine provisioning state</t>
+        </is>
+      </c>
+      <c r="F178" s="4" t="n"/>
+      <c r="G178" s="4" t="n"/>
+      <c r="H178" s="4" t="n"/>
+      <c r="I178" s="4" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="4" t="inlineStr">
+        <is>
+          <t>TC-1124</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>Force bypasses state check</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+        </is>
+      </c>
+      <c r="E179" s="4" t="inlineStr">
+        <is>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
+        </is>
+      </c>
+      <c r="F179" s="4" t="n"/>
+      <c r="G179" s="4" t="n"/>
+      <c r="H179" s="4" t="n"/>
+      <c r="I179" s="4" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>TC-1125</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>Unmigrated DB treated as initial setup</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t>200, request allowed (not 503)</t>
+        </is>
+      </c>
+      <c r="F180" s="4" t="n"/>
+      <c r="G180" s="4" t="n"/>
+      <c r="H180" s="4" t="n"/>
+      <c r="I180" s="4" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>TC-1126</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t>Fresh install — DB/role missing</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+        </is>
+      </c>
+      <c r="E181" s="4" t="inlineStr">
+        <is>
+          <t>200, provisioning proceeds (not 503)</t>
+        </is>
+      </c>
+      <c r="F181" s="4" t="n"/>
+      <c r="G181" s="4" t="n"/>
+      <c r="H181" s="4" t="n"/>
+      <c r="I181" s="4" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="4" t="inlineStr">
+        <is>
+          <t>TC-1127</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C182" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — OperationalError on reachable DB</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E182" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F182" s="4" t="n"/>
+      <c r="G182" s="4" t="n"/>
+      <c r="H182" s="4" t="n"/>
+      <c r="I182" s="4" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="4" t="inlineStr">
+        <is>
+          <t>TC-1128</t>
+        </is>
+      </c>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C183" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — unexpected error</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E183" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F183" s="4" t="n"/>
+      <c r="G183" s="4" t="n"/>
+      <c r="H183" s="4" t="n"/>
+      <c r="I183" s="4" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="4" t="inlineStr">
+        <is>
+          <t>TC-1129</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C184" s="4" t="inlineStr">
+        <is>
+          <t>Provision — migration failure</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+        </is>
+      </c>
+      <c r="E184" s="4" t="inlineStr">
+        <is>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+        </is>
+      </c>
+      <c r="F184" s="4" t="n"/>
+      <c r="G184" s="4" t="n"/>
+      <c r="H184" s="4" t="n"/>
+      <c r="I184" s="4" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="4" t="inlineStr">
+        <is>
+          <t>TC-1130</t>
+        </is>
+      </c>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C185" s="4" t="inlineStr">
+        <is>
+          <t>Provision — .env write failure</t>
+        </is>
+      </c>
+      <c r="D185" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+        </is>
+      </c>
+      <c r="E185" s="4" t="inlineStr">
+        <is>
+          <t>500, "failed to persist" message; engine not swapped</t>
+        </is>
+      </c>
+      <c r="F185" s="4" t="n"/>
+      <c r="G185" s="4" t="n"/>
+      <c r="H185" s="4" t="n"/>
+      <c r="I185" s="4" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>TC-1131</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>Provision — engine reinit failure</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>500, "engine could not be switched" message; .env already written</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="n"/>
+      <c r="G186" s="4" t="n"/>
+      <c r="H186" s="4" t="n"/>
+      <c r="I186" s="4" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B171" s="5" t="n">
-        <v>155</v>
+      <c r="B188" s="5" t="n">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update documentation to reflect port enablement behavior changes and audit log details
</commit_message>
<xml_diff>
--- a/documents/testing/ecube-qa-test-cases.xlsx
+++ b/documents/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I188"/>
+  <dimension ref="A1:I190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2512,17 +2512,17 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>PORT_ENABLED audit log</t>
+          <t>Disable port — AVAILABLE drive demoted</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=PORT_ENABLED after enabling a port</t>
+          <t>Enable port, confirm drive is AVAILABLE, disable port, run POST /drives/refresh</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with port_id, system_path, hub_id</t>
+          <t>Drive transitions to EMPTY</t>
         </is>
       </c>
       <c r="F73" s="4" t="n"/>
@@ -2543,17 +2543,17 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>PORT_DISABLED audit log</t>
+          <t>Orphan drive stays EMPTY</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=PORT_DISABLED after disabling a port</t>
+          <t>Discover a drive with no matching port (port_id = NULL), run POST /drives/refresh</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with port_id, system_path, hub_id</t>
+          <t>Drive remains in EMPTY state (unknown port treated as disabled)</t>
         </is>
       </c>
       <c r="F74" s="4" t="n"/>
@@ -2562,48 +2562,60 @@
       <c r="I74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>§12.5 USB Hardware</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>12.5 USB Hardware</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="n"/>
-      <c r="D75" s="3" t="n"/>
-      <c r="E75" s="3" t="n"/>
-      <c r="F75" s="3" t="n"/>
-      <c r="G75" s="3" t="n"/>
-      <c r="H75" s="3" t="n"/>
-      <c r="I75" s="3" t="n"/>
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>TC-446</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>12.4.3 Port Enablement</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>PORT_ENABLED audit log</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=PORT_ENABLED after enabling a port</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Audit entry with port_id, system_path, hub_id, enabled, path</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="n"/>
+      <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>TC-501</t>
+          <t>TC-447</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.3 Port Enablement</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Hot-plug detection</t>
+          <t>PORT_DISABLED audit log</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>Plug in a USB drive, wait 30 seconds</t>
+          <t>GET /audit?action=PORT_DISABLED after disabling a port</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>GET /drives shows the new drive (in EMPTY state if port is disabled, or AVAILABLE if port is enabled)</t>
+          <t>Audit entry with port_id, system_path, hub_id, enabled, path</t>
         </is>
       </c>
       <c r="F76" s="4" t="n"/>
@@ -2612,40 +2624,28 @@
       <c r="I76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>TC-502</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>§12.5 USB Hardware</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>USB topology</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>GET /introspection/usb/topology</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>Shows real hub serial numbers, port numbers, connected devices</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="n"/>
-      <c r="G77" s="4" t="n"/>
-      <c r="H77" s="4" t="n"/>
-      <c r="I77" s="4" t="n"/>
+      <c r="C77" s="3" t="n"/>
+      <c r="D77" s="3" t="n"/>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
+      <c r="G77" s="3" t="n"/>
+      <c r="H77" s="3" t="n"/>
+      <c r="I77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>TC-503</t>
+          <t>TC-501</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -2655,17 +2655,17 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Physical eject</t>
+          <t>Hot-plug detection</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Initialize drive → prepare-eject → physically remove</t>
+          <t>Plug in a USB drive, wait 30 seconds</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
+          <t>GET /drives shows the new drive (in EMPTY state if port is disabled, or AVAILABLE if port is enabled)</t>
         </is>
       </c>
       <c r="F78" s="4" t="n"/>
@@ -2676,7 +2676,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>TC-504</t>
+          <t>TC-502</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
@@ -2686,17 +2686,17 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Re-plug same drive</t>
+          <t>USB topology</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>Remove and re-insert the same drive</t>
+          <t>GET /introspection/usb/topology</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
+          <t>Shows real hub serial numbers, port numbers, connected devices</t>
         </is>
       </c>
       <c r="F79" s="4" t="n"/>
@@ -2707,7 +2707,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>TC-505</t>
+          <t>TC-503</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
@@ -2717,17 +2717,17 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Multiple drives</t>
+          <t>Physical eject</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Plug in 2+ drives simultaneously</t>
+          <t>Initialize drive → prepare-eject → physically remove</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>All drives appear in /drives; each can be initialized to different projects</t>
+          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
         </is>
       </c>
       <c r="F80" s="4" t="n"/>
@@ -2738,7 +2738,7 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>TC-506</t>
+          <t>TC-504</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -2748,17 +2748,17 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Sync + unmount</t>
+          <t>Re-plug same drive</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Initialize drive, create/start a job, then prepare-eject</t>
+          <t>Remove and re-insert the same drive</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
+          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
         </is>
       </c>
       <c r="F81" s="4" t="n"/>
@@ -2769,7 +2769,7 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>TC-507</t>
+          <t>TC-505</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -2779,17 +2779,17 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Disabled port blocks AVAILABLE</t>
+          <t>Multiple drives</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Disable a port, plug in a drive to that port, run discovery</t>
+          <t>Plug in 2+ drives simultaneously</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Drive appears in EMPTY state; enable port + refresh → drive transitions to AVAILABLE</t>
+          <t>All drives appear in /drives; each can be initialized to different projects</t>
         </is>
       </c>
       <c r="F82" s="4" t="n"/>
@@ -2798,48 +2798,60 @@
       <c r="I82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>§12.6 End-to-End Copy</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>12.6 End-to-End Copy</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="n"/>
-      <c r="D83" s="3" t="n"/>
-      <c r="E83" s="3" t="n"/>
-      <c r="F83" s="3" t="n"/>
-      <c r="G83" s="3" t="n"/>
-      <c r="H83" s="3" t="n"/>
-      <c r="I83" s="3" t="n"/>
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>TC-506</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>12.5 USB Hardware</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Sync + unmount</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Initialize drive, create/start a job, then prepare-eject</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="n"/>
+      <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>TC-601</t>
+          <t>TC-507</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>12.6 End-to-End Copy</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Full E2E workflow</t>
+          <t>Disabled port blocks AVAILABLE</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Setup test files → add mount → discover drive → initialize → create job → start → poll → verify → manifest → eject → verify on another machine</t>
+          <t>Disable a port, plug in a drive to that port, run discovery</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>All steps succeed; checksums match; audit trail shows complete chain</t>
+          <t>Drive appears in EMPTY state; enable port + refresh → drive transitions to AVAILABLE</t>
         </is>
       </c>
       <c r="F84" s="4" t="n"/>
@@ -2850,12 +2862,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>§12.7 Error Handling</t>
+          <t>§12.6 End-to-End Copy</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.6 End-to-End Copy</t>
         </is>
       </c>
       <c r="C85" s="3" t="n"/>
@@ -2869,23 +2881,27 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>TC-701</t>
+          <t>TC-601</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.6 End-to-End Copy</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/99999</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr"/>
+          <t>Full E2E workflow</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Setup test files → add mount → discover drive → initialize → create job → start → poll → verify → manifest → eject → verify on another machine</t>
+        </is>
+      </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>All steps succeed; checksums match; audit trail shows complete chain</t>
         </is>
       </c>
       <c r="F86" s="4" t="n"/>
@@ -2894,36 +2910,28 @@
       <c r="I86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="inlineStr">
-        <is>
-          <t>TC-702</t>
-        </is>
-      </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>§12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>12.7 Error Handling</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
-        <is>
-          <t>DELETE /mounts/99999</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr"/>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>404, NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="F87" s="4" t="n"/>
-      <c r="G87" s="4" t="n"/>
-      <c r="H87" s="4" t="n"/>
-      <c r="I87" s="4" t="n"/>
+      <c r="C87" s="3" t="n"/>
+      <c r="D87" s="3" t="n"/>
+      <c r="E87" s="3" t="n"/>
+      <c r="F87" s="3" t="n"/>
+      <c r="G87" s="3" t="n"/>
+      <c r="H87" s="3" t="n"/>
+      <c r="I87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>TC-703</t>
+          <t>TC-701</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
@@ -2933,13 +2941,13 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Start an already-running job</t>
+          <t>GET /jobs/99999</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr"/>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>409, CONFLICT</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F88" s="4" t="n"/>
@@ -2950,7 +2958,7 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>TC-704</t>
+          <t>TC-702</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
@@ -2960,13 +2968,13 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>All error responses</t>
+          <t>DELETE /mounts/99999</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr"/>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>JSON body includes code, message, and trace_id</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F89" s="4" t="n"/>
@@ -2977,7 +2985,7 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>TC-705</t>
+          <t>TC-703</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
@@ -2987,13 +2995,13 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/999/format with {"filesystem_type": "ext4"}</t>
+          <t>Start an already-running job</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr"/>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>409, CONFLICT</t>
         </is>
       </c>
       <c r="F90" s="4" t="n"/>
@@ -3004,7 +3012,7 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>TC-706</t>
+          <t>TC-704</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
@@ -3014,13 +3022,13 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
+          <t>All error responses</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr"/>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>422, validation error</t>
+          <t>JSON body includes code, message, and trace_id</t>
         </is>
       </c>
       <c r="F91" s="4" t="n"/>
@@ -3031,7 +3039,7 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>TC-707</t>
+          <t>TC-705</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
@@ -3041,13 +3049,13 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with empty body</t>
+          <t>POST /drives/999/format with {"filesystem_type": "ext4"}</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr"/>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F92" s="4" t="n"/>
@@ -3056,48 +3064,52 @@
       <c r="I92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>§12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="n"/>
-      <c r="D93" s="3" t="n"/>
-      <c r="E93" s="3" t="n"/>
-      <c r="F93" s="3" t="n"/>
-      <c r="G93" s="3" t="n"/>
-      <c r="H93" s="3" t="n"/>
-      <c r="I93" s="3" t="n"/>
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>TC-706</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr"/>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>422, validation error</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="n"/>
+      <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
+      <c r="I93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>TC-801</t>
+          <t>TC-707</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>List users (empty)</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>GET /users with admin token (no roles assigned yet)</t>
-        </is>
-      </c>
+          <t>POST /drives/{id}/format with empty body</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr"/>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>200, {"users": []}</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F94" s="4" t="n"/>
@@ -3106,40 +3118,28 @@
       <c r="I94" s="4" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="inlineStr">
-        <is>
-          <t>TC-802</t>
-        </is>
-      </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>§12.8 User Role Mgmt</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
-        <is>
-          <t>Assign roles</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["processor", "auditor"]}</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>200, returns username and sorted roles</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="n"/>
-      <c r="G95" s="4" t="n"/>
-      <c r="H95" s="4" t="n"/>
-      <c r="I95" s="4" t="n"/>
+      <c r="C95" s="3" t="n"/>
+      <c r="D95" s="3" t="n"/>
+      <c r="E95" s="3" t="n"/>
+      <c r="F95" s="3" t="n"/>
+      <c r="G95" s="3" t="n"/>
+      <c r="H95" s="3" t="n"/>
+      <c r="I95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>TC-803</t>
+          <t>TC-801</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -3149,17 +3149,17 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Get roles</t>
+          <t>List users (empty)</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>GET /users/qa-processor/roles after assignment</t>
+          <t>GET /users with admin token (no roles assigned yet)</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
+          <t>200, {"users": []}</t>
         </is>
       </c>
       <c r="F96" s="4" t="n"/>
@@ -3170,7 +3170,7 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>TC-804</t>
+          <t>TC-802</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
@@ -3180,17 +3180,17 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>List users after assignment</t>
+          <t>Assign roles</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>GET /users after assigning roles</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["processor", "auditor"]}</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>200, user appears in list with correct roles</t>
+          <t>200, returns username and sorted roles</t>
         </is>
       </c>
       <c r="F97" s="4" t="n"/>
@@ -3201,7 +3201,7 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>TC-805</t>
+          <t>TC-803</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
@@ -3211,17 +3211,17 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Replace roles</t>
+          <t>Get roles</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["manager"]}</t>
+          <t>GET /users/qa-processor/roles after assignment</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>200, only ["manager"] returned; old roles removed</t>
+          <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
         </is>
       </c>
       <c r="F98" s="4" t="n"/>
@@ -3232,7 +3232,7 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>TC-806</t>
+          <t>TC-804</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
@@ -3242,17 +3242,17 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Deduplicate roles</t>
+          <t>List users after assignment</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
+          <t>GET /users after assigning roles</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>200, deduplicated to ["admin", "processor"]</t>
+          <t>200, user appears in list with correct roles</t>
         </is>
       </c>
       <c r="F99" s="4" t="n"/>
@@ -3263,7 +3263,7 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>TC-807</t>
+          <t>TC-805</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
@@ -3273,17 +3273,17 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Invalid role name</t>
+          <t>Replace roles</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["manager"]}</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>422, error message mentions superuser</t>
+          <t>200, only ["manager"] returned; old roles removed</t>
         </is>
       </c>
       <c r="F100" s="4" t="n"/>
@@ -3294,7 +3294,7 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>TC-808</t>
+          <t>TC-806</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
@@ -3304,17 +3304,17 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Empty role list</t>
+          <t>Deduplicate roles</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>422, at least one role required</t>
+          <t>200, deduplicated to ["admin", "processor"]</t>
         </is>
       </c>
       <c r="F101" s="4" t="n"/>
@@ -3325,7 +3325,7 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>TC-809</t>
+          <t>TC-807</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
@@ -3335,17 +3335,17 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Remove roles</t>
+          <t>Invalid role name</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>DELETE /users/qa-processor/roles</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "qa-processor", "roles": []}</t>
+          <t>422, error message mentions superuser</t>
         </is>
       </c>
       <c r="F102" s="4" t="n"/>
@@ -3356,7 +3356,7 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>TC-810</t>
+          <t>TC-808</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
@@ -3366,17 +3366,17 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>Get roles after removal</t>
+          <t>Empty role list</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>GET /users/qa-processor/roles after DELETE</t>
+          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
         </is>
       </c>
       <c r="E103" s="4" t="inlineStr">
         <is>
-          <t>200, {"roles": []}</t>
+          <t>422, at least one role required</t>
         </is>
       </c>
       <c r="F103" s="4" t="n"/>
@@ -3387,7 +3387,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>TC-811</t>
+          <t>TC-809</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
@@ -3397,17 +3397,17 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Get roles for unknown user</t>
+          <t>Remove roles</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>GET /users/nonexistent/roles</t>
+          <t>DELETE /users/qa-processor/roles</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "nonexistent", "roles": []}</t>
+          <t>200, {"username": "qa-processor", "roles": []}</t>
         </is>
       </c>
       <c r="F104" s="4" t="n"/>
@@ -3418,7 +3418,7 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>TC-812</t>
+          <t>TC-810</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
@@ -3428,17 +3428,17 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot list users</t>
+          <t>Get roles after removal</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>GET /users with processor token</t>
+          <t>GET /users/qa-processor/roles after DELETE</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, {"roles": []}</t>
         </is>
       </c>
       <c r="F105" s="4" t="n"/>
@@ -3449,7 +3449,7 @@
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>TC-813</t>
+          <t>TC-811</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
@@ -3459,17 +3459,17 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot set roles</t>
+          <t>Get roles for unknown user</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/x/roles with processor token</t>
+          <t>GET /users/nonexistent/roles</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>200, {"username": "nonexistent", "roles": []}</t>
         </is>
       </c>
       <c r="F106" s="4" t="n"/>
@@ -3480,7 +3480,7 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>TC-814</t>
+          <t>TC-812</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
@@ -3490,12 +3490,12 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot delete roles</t>
+          <t>Processor cannot list users</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>DELETE /users/x/roles with processor token</t>
+          <t>GET /users with processor token</t>
         </is>
       </c>
       <c r="E107" s="4" t="inlineStr">
@@ -3511,7 +3511,7 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>TC-815</t>
+          <t>TC-813</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated access</t>
+          <t>Processor cannot set roles</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>GET /users without Authorization header</t>
+          <t>PUT /users/x/roles with processor token</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F108" s="4" t="n"/>
@@ -3542,7 +3542,7 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>TC-816</t>
+          <t>TC-814</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
@@ -3552,17 +3552,17 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>ROLE_ASSIGNED audit log</t>
+          <t>Processor cannot delete roles</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=ROLE_ASSIGNED after assigning roles</t>
+          <t>DELETE /users/x/roles with processor token</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor, target user, and roles</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F109" s="4" t="n"/>
@@ -3573,7 +3573,7 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>TC-817</t>
+          <t>TC-815</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
@@ -3583,17 +3583,17 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>ROLE_REMOVED audit log</t>
+          <t>Unauthenticated access</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=ROLE_REMOVED after removing roles</t>
+          <t>GET /users without Authorization header</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and target user</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F110" s="4" t="n"/>
@@ -3604,7 +3604,7 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>TC-818</t>
+          <t>TC-816</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
@@ -3614,17 +3614,17 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>DB roles override groups</t>
+          <t>ROLE_ASSIGNED audit log</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
+          <t>GET /audit?action=ROLE_ASSIGNED after assigning roles</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
+          <t>Audit entry with actor, target user, and roles</t>
         </is>
       </c>
       <c r="F111" s="4" t="n"/>
@@ -3635,7 +3635,7 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>TC-819</t>
+          <t>TC-817</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
@@ -3645,17 +3645,17 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>Fallback to group roles</t>
+          <t>ROLE_REMOVED audit log</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
+          <t>GET /audit?action=ROLE_REMOVED after removing roles</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>JWT roles falls back to OS group mapping (["processor"])</t>
+          <t>Audit entry with actor and target user</t>
         </is>
       </c>
       <c r="F112" s="4" t="n"/>
@@ -3664,48 +3664,60 @@
       <c r="I112" s="4" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>§12.9 OS User &amp; Group Mgmt</t>
-        </is>
-      </c>
-      <c r="B113" s="2" t="inlineStr">
-        <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="n"/>
-      <c r="D113" s="3" t="n"/>
-      <c r="E113" s="3" t="n"/>
-      <c r="F113" s="3" t="n"/>
-      <c r="G113" s="3" t="n"/>
-      <c r="H113" s="3" t="n"/>
-      <c r="I113" s="3" t="n"/>
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>TC-818</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>12.8 User Role Mgmt</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>DB roles override groups</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>TC-901</t>
+          <t>TC-819</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Create group</t>
+          <t>Fallback to group roles</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
+          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>201, returns name, gid, members</t>
+          <t>JWT roles falls back to OS group mapping (["processor"])</t>
         </is>
       </c>
       <c r="F114" s="4" t="n"/>
@@ -3714,40 +3726,28 @@
       <c r="I114" s="4" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="4" t="inlineStr">
-        <is>
-          <t>TC-902</t>
-        </is>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>§12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C115" s="4" t="inlineStr">
-        <is>
-          <t>Create group without prefix</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr">
-        <is>
-          <t>POST /admin/os-groups with {"name": "testers"}</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="inlineStr">
-        <is>
-          <t>422, group name must start with ecube-</t>
-        </is>
-      </c>
-      <c r="F115" s="4" t="n"/>
-      <c r="G115" s="4" t="n"/>
-      <c r="H115" s="4" t="n"/>
-      <c r="I115" s="4" t="n"/>
+      <c r="C115" s="3" t="n"/>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="3" t="n"/>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="3" t="n"/>
+      <c r="I115" s="3" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>TC-903</t>
+          <t>TC-901</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
@@ -3757,17 +3757,17 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>List groups</t>
+          <t>Create group</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-groups</t>
+          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>200, only ecube-* groups listed</t>
+          <t>201, returns name, gid, members</t>
         </is>
       </c>
       <c r="F116" s="4" t="n"/>
@@ -3778,7 +3778,7 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>TC-904</t>
+          <t>TC-902</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -3788,17 +3788,17 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Delete group</t>
+          <t>Create group without prefix</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-groups/ecube-testers</t>
+          <t>POST /admin/os-groups with {"name": "testers"}</t>
         </is>
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>422, group name must start with ecube-</t>
         </is>
       </c>
       <c r="F117" s="4" t="n"/>
@@ -3809,7 +3809,7 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>TC-905</t>
+          <t>TC-903</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
@@ -3819,17 +3819,17 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>Delete group without prefix</t>
+          <t>List groups</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-groups/somegroup</t>
+          <t>GET /admin/os-groups</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>422, group name must start with ecube-</t>
+          <t>200, only ecube-* groups listed</t>
         </is>
       </c>
       <c r="F118" s="4" t="n"/>
@@ -3840,7 +3840,7 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>TC-906</t>
+          <t>TC-904</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
@@ -3850,17 +3850,17 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Create user</t>
+          <t>Delete group</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with username, password, groups, roles</t>
+          <t>DELETE /admin/os-groups/ecube-testers</t>
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>201, returns username, uid, gid, home, shell, groups</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F119" s="4" t="n"/>
@@ -3871,7 +3871,7 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>TC-907</t>
+          <t>TC-905</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Create user — duplicate</t>
+          <t>Delete group without prefix</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with existing username</t>
+          <t>DELETE /admin/os-groups/somegroup</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>422, group name must start with ecube-</t>
         </is>
       </c>
       <c r="F120" s="4" t="n"/>
@@ -3902,7 +3902,7 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>TC-908</t>
+          <t>TC-906</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
@@ -3912,17 +3912,17 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Create user — reserved name</t>
+          <t>Create user</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"username": "root", ...}</t>
+          <t>POST /admin/os-users with username, password, groups, roles</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>422, reserved username</t>
+          <t>201, returns username, uid, gid, home, shell, groups</t>
         </is>
       </c>
       <c r="F121" s="4" t="n"/>
@@ -3933,7 +3933,7 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>TC-909</t>
+          <t>TC-907</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
@@ -3943,17 +3943,17 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Create user — empty password</t>
+          <t>Create user — duplicate</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"password": "", ...}</t>
+          <t>POST /admin/os-users with existing username</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F122" s="4" t="n"/>
@@ -3964,7 +3964,7 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>TC-910</t>
+          <t>TC-908</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
@@ -3974,17 +3974,17 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with newline</t>
+          <t>Create user — reserved name</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing \n</t>
+          <t>POST /admin/os-users with {"username": "root", ...}</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422, reserved username</t>
         </is>
       </c>
       <c r="F123" s="4" t="n"/>
@@ -3995,7 +3995,7 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>TC-911</t>
+          <t>TC-909</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
@@ -4005,17 +4005,17 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with colon</t>
+          <t>Create user — empty password</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing :</t>
+          <t>POST /admin/os-users with {"password": "", ...}</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F124" s="4" t="n"/>
@@ -4026,7 +4026,7 @@
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>TC-912</t>
+          <t>TC-910</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
@@ -4036,17 +4036,17 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Create user — invalid group</t>
+          <t>Create user — password with newline</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with non-existent group in groups list</t>
+          <t>POST /admin/os-users with password containing \n</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>422, group does not exist</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F125" s="4" t="n"/>
@@ -4057,7 +4057,7 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>TC-913</t>
+          <t>TC-911</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
@@ -4067,17 +4067,17 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Create user — no ecube-* group</t>
+          <t>Create user — password with colon</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
+          <t>POST /admin/os-users with password containing :</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F126" s="4" t="n"/>
@@ -4088,7 +4088,7 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>TC-914</t>
+          <t>TC-912</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
@@ -4098,17 +4098,17 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>List users</t>
+          <t>Create user — invalid group</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users</t>
+          <t>POST /admin/os-users with non-existent group in groups list</t>
         </is>
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>200, only users in ecube-* groups listed</t>
+          <t>422, group does not exist</t>
         </is>
       </c>
       <c r="F127" s="4" t="n"/>
@@ -4119,7 +4119,7 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>TC-915</t>
+          <t>TC-913</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
@@ -4129,17 +4129,17 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Reset password</t>
+          <t>Create user — no ecube-* group</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F128" s="4" t="n"/>
@@ -4150,7 +4150,7 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>TC-916</t>
+          <t>TC-914</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
@@ -4160,17 +4160,17 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Reset password — non-ECUBE user</t>
+          <t>List users</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/postgres/password</t>
+          <t>GET /admin/os-users</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200, only users in ecube-* groups listed</t>
         </is>
       </c>
       <c r="F129" s="4" t="n"/>
@@ -4181,7 +4181,7 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>TC-917</t>
+          <t>TC-915</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
@@ -4191,17 +4191,17 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Replace groups</t>
+          <t>Reset password</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
+          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list; non-ecube-* groups preserved</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F130" s="4" t="n"/>
@@ -4212,7 +4212,7 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>TC-918</t>
+          <t>TC-916</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
@@ -4222,17 +4222,17 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — empty list</t>
+          <t>Reset password — non-ECUBE user</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
+          <t>PUT /admin/os-users/postgres/password</t>
         </is>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F131" s="4" t="n"/>
@@ -4243,7 +4243,7 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>TC-919</t>
+          <t>TC-917</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
@@ -4253,17 +4253,17 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — non-ecube name</t>
+          <t>Replace groups</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>422, group does not start with ecube-</t>
+          <t>200, updated group list; non-ecube-* groups preserved</t>
         </is>
       </c>
       <c r="F132" s="4" t="n"/>
@@ -4274,7 +4274,7 @@
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
         <is>
-          <t>TC-920</t>
+          <t>TC-918</t>
         </is>
       </c>
       <c r="B133" s="4" t="inlineStr">
@@ -4284,17 +4284,17 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>Append groups</t>
+          <t>Replace groups — empty list</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
         </is>
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F133" s="4" t="n"/>
@@ -4305,7 +4305,7 @@
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>TC-921</t>
+          <t>TC-919</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -4315,17 +4315,17 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Modify groups — non-ECUBE user</t>
+          <t>Replace groups — non-ecube name</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/www-data/groups</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>422, group does not start with ecube-</t>
         </is>
       </c>
       <c r="F134" s="4" t="n"/>
@@ -4336,7 +4336,7 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>TC-922</t>
+          <t>TC-920</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -4346,17 +4346,17 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Delete user</t>
+          <t>Append groups</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/{username}</t>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>200, user and DB roles removed</t>
+          <t>200, updated group list</t>
         </is>
       </c>
       <c r="F135" s="4" t="n"/>
@@ -4367,7 +4367,7 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>TC-923</t>
+          <t>TC-921</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -4377,12 +4377,12 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Delete user — non-ECUBE user</t>
+          <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/daemon</t>
+          <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
@@ -4398,7 +4398,7 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>TC-924</t>
+          <t>TC-922</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -4408,17 +4408,17 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Delete user — not found</t>
+          <t>Delete user</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/nonexistent</t>
+          <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200, user and DB roles removed</t>
         </is>
       </c>
       <c r="F137" s="4" t="n"/>
@@ -4429,7 +4429,7 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>TC-925</t>
+          <t>TC-923</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -4439,17 +4439,17 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot access OS endpoints</t>
+          <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users with processor token</t>
+          <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F138" s="4" t="n"/>
@@ -4460,7 +4460,7 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>TC-926</t>
+          <t>TC-924</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -4470,17 +4470,17 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Non-local mode returns 404</t>
+          <t>Delete user — not found</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+          <t>DELETE /admin/os-users/nonexistent</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>404, Not Found</t>
+          <t>404</t>
         </is>
       </c>
       <c r="F139" s="4" t="n"/>
@@ -4491,7 +4491,7 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>TC-927</t>
+          <t>TC-925</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -4501,17 +4501,17 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_CREATED audit log</t>
+          <t>Processor cannot access OS endpoints</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+          <t>GET /admin/os-users with processor token</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F140" s="4" t="n"/>
@@ -4522,7 +4522,7 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>TC-928</t>
+          <t>TC-926</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -4532,17 +4532,17 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_DELETED audit log</t>
+          <t>Non-local mode returns 404</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>404, Not Found</t>
         </is>
       </c>
       <c r="F141" s="4" t="n"/>
@@ -4553,7 +4553,7 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>TC-929</t>
+          <t>TC-927</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -4563,17 +4563,17 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>OS_PASSWORD_RESET audit log</t>
+          <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>Audit entry (no password in details)</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F142" s="4" t="n"/>
@@ -4584,7 +4584,7 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>TC-930</t>
+          <t>TC-928</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -4594,17 +4594,17 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_CREATED audit log</t>
+          <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F143" s="4" t="n"/>
@@ -4615,7 +4615,7 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>TC-931</t>
+          <t>TC-929</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -4625,17 +4625,17 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_DELETED audit log</t>
+          <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>Audit entry (no password in details)</t>
         </is>
       </c>
       <c r="F144" s="4" t="n"/>
@@ -4644,48 +4644,60 @@
       <c r="I144" s="4" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="inlineStr">
-        <is>
-          <t>§12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B145" s="2" t="inlineStr">
-        <is>
-          <t>12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C145" s="3" t="n"/>
-      <c r="D145" s="3" t="n"/>
-      <c r="E145" s="3" t="n"/>
-      <c r="F145" s="3" t="n"/>
-      <c r="G145" s="3" t="n"/>
-      <c r="H145" s="3" t="n"/>
-      <c r="I145" s="3" t="n"/>
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>TC-930</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>OS_GROUP_CREATED audit log</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="inlineStr">
+        <is>
+          <t>Audit entry with group name</t>
+        </is>
+      </c>
+      <c r="F145" s="4" t="n"/>
+      <c r="G145" s="4" t="n"/>
+      <c r="H145" s="4" t="n"/>
+      <c r="I145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>TC-1001</t>
+          <t>TC-931</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>OS_GROUP_DELETED audit log</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F146" s="4" t="n"/>
@@ -4694,40 +4706,28 @@
       <c r="I146" s="4" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="4" t="inlineStr">
-        <is>
-          <t>TC-1002</t>
-        </is>
-      </c>
-      <c r="B147" s="4" t="inlineStr">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>§12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C147" s="4" t="inlineStr">
-        <is>
-          <t>Initialize</t>
-        </is>
-      </c>
-      <c r="D147" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/initialize with valid username and password</t>
-        </is>
-      </c>
-      <c r="E147" s="4" t="inlineStr">
-        <is>
-          <t>200, returns message, username, groups_created</t>
-        </is>
-      </c>
-      <c r="F147" s="4" t="n"/>
-      <c r="G147" s="4" t="n"/>
-      <c r="H147" s="4" t="n"/>
-      <c r="I147" s="4" t="n"/>
+      <c r="C147" s="3" t="n"/>
+      <c r="D147" s="3" t="n"/>
+      <c r="E147" s="3" t="n"/>
+      <c r="F147" s="3" t="n"/>
+      <c r="G147" s="3" t="n"/>
+      <c r="H147" s="3" t="n"/>
+      <c r="I147" s="3" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
@@ -4737,17 +4737,17 @@
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F148" s="4" t="n"/>
@@ -4758,7 +4758,7 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
@@ -4768,17 +4768,17 @@
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>
@@ -4789,7 +4789,7 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
@@ -4799,17 +4799,17 @@
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F150" s="4" t="n"/>
@@ -4820,7 +4820,7 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
@@ -4830,17 +4830,17 @@
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F151" s="4" t="n"/>
@@ -4851,7 +4851,7 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
@@ -4861,17 +4861,17 @@
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F152" s="4" t="n"/>
@@ -4882,7 +4882,7 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
@@ -4892,17 +4892,17 @@
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F153" s="4" t="n"/>
@@ -4913,7 +4913,7 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
@@ -4923,17 +4923,17 @@
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F154" s="4" t="n"/>
@@ -4942,48 +4942,60 @@
       <c r="I154" s="4" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C155" s="3" t="n"/>
-      <c r="D155" s="3" t="n"/>
-      <c r="E155" s="3" t="n"/>
-      <c r="F155" s="3" t="n"/>
-      <c r="G155" s="3" t="n"/>
-      <c r="H155" s="3" t="n"/>
-      <c r="I155" s="3" t="n"/>
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>TC-1008</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Login as initialized admin</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/token with the admin credentials from step 2</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>200, JWT contains admin role</t>
+        </is>
+      </c>
+      <c r="F155" s="4" t="n"/>
+      <c r="G155" s="4" t="n"/>
+      <c r="H155" s="4" t="n"/>
+      <c r="I155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-1009</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>Test connection — success</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "ok", "server_version": "..."}</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F156" s="4" t="n"/>
@@ -4992,40 +5004,28 @@
       <c r="I156" s="4" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="4" t="inlineStr">
-        <is>
-          <t>TC-1102</t>
-        </is>
-      </c>
-      <c r="B157" s="4" t="inlineStr">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C157" s="4" t="inlineStr">
-        <is>
-          <t>Test connection — bad host</t>
-        </is>
-      </c>
-      <c r="D157" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/database/test-connection with unreachable host</t>
-        </is>
-      </c>
-      <c r="E157" s="4" t="inlineStr">
-        <is>
-          <t>400, connection error</t>
-        </is>
-      </c>
-      <c r="F157" s="4" t="n"/>
-      <c r="G157" s="4" t="n"/>
-      <c r="H157" s="4" t="n"/>
-      <c r="I157" s="4" t="n"/>
+      <c r="C157" s="3" t="n"/>
+      <c r="D157" s="3" t="n"/>
+      <c r="E157" s="3" t="n"/>
+      <c r="F157" s="3" t="n"/>
+      <c r="G157" s="3" t="n"/>
+      <c r="H157" s="3" t="n"/>
+      <c r="I157" s="3" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
@@ -5035,17 +5035,17 @@
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Test connection — SSRF host</t>
+          <t>Test connection — success</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>422, invalid host</t>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
       <c r="F158" s="4" t="n"/>
@@ -5056,7 +5056,7 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
@@ -5066,17 +5066,17 @@
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Test connection — port out of range</t>
+          <t>Test connection — bad host</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "port": 99999</t>
+          <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F159" s="4" t="n"/>
@@ -5087,7 +5087,7 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
@@ -5097,17 +5097,17 @@
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Provision — success</t>
+          <t>Test connection — SSRF host</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials</t>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>422, invalid host</t>
         </is>
       </c>
       <c r="F160" s="4" t="n"/>
@@ -5118,7 +5118,7 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
@@ -5128,17 +5128,17 @@
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Provision — bad admin credentials</t>
+          <t>Test connection — port out of range</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with wrong admin password</t>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F161" s="4" t="n"/>
@@ -5149,7 +5149,7 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
@@ -5159,17 +5159,17 @@
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Provision — invalid database name</t>
+          <t>Provision — success</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
+          <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>422, invalid identifier</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F162" s="4" t="n"/>
@@ -5180,7 +5180,7 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>TC-1108</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
@@ -5190,17 +5190,17 @@
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Status — connected</t>
+          <t>Provision — bad admin credentials</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with admin token</t>
+          <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>200, connected: true, migration info</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F163" s="4" t="n"/>
@@ -5211,7 +5211,7 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
@@ -5221,17 +5221,17 @@
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Status — requires auth</t>
+          <t>Provision — invalid database name</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status without token</t>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>422, invalid identifier</t>
         </is>
       </c>
       <c r="F164" s="4" t="n"/>
@@ -5242,7 +5242,7 @@
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B165" s="4" t="inlineStr">
@@ -5252,17 +5252,17 @@
       </c>
       <c r="C165" s="4" t="inlineStr">
         <is>
-          <t>Status — requires admin</t>
+          <t>Status — connected</t>
         </is>
       </c>
       <c r="D165" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with processor token</t>
+          <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
       <c r="E165" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>200, connected: true, migration info</t>
         </is>
       </c>
       <c r="F165" s="4" t="n"/>
@@ -5273,7 +5273,7 @@
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
@@ -5283,17 +5283,17 @@
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Settings update — success</t>
+          <t>Status — requires auth</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with valid partial update</t>
+          <t>GET /setup/database/status without token</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "updated", ...}</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F166" s="4" t="n"/>
@@ -5304,7 +5304,7 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
@@ -5314,17 +5314,17 @@
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Settings update — bad connection</t>
+          <t>Status — requires admin</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with unreachable host</t>
+          <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>400, connection test failed</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F167" s="4" t="n"/>
@@ -5335,7 +5335,7 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
@@ -5345,17 +5345,17 @@
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Settings update — empty body</t>
+          <t>Settings update — success</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with {}</t>
+          <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>422, at least one field required</t>
+          <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
       <c r="F168" s="4" t="n"/>
@@ -5366,7 +5366,7 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
@@ -5376,17 +5376,17 @@
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Settings update — requires admin</t>
+          <t>Settings update — bad connection</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with processor token</t>
+          <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>400, connection test failed</t>
         </is>
       </c>
       <c r="F169" s="4" t="n"/>
@@ -5397,7 +5397,7 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
@@ -5407,17 +5407,17 @@
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — test-connection</t>
+          <t>Settings update — empty body</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+          <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>422, at least one field required</t>
         </is>
       </c>
       <c r="F170" s="4" t="n"/>
@@ -5428,7 +5428,7 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>TC-1116</t>
+          <t>TC-1114</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
@@ -5438,17 +5438,17 @@
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — provision</t>
+          <t>Settings update — requires admin</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision without token (after admin exists)</t>
+          <t>PUT /setup/database/settings with processor token</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F171" s="4" t="n"/>
@@ -5459,7 +5459,7 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>TC-1117</t>
+          <t>TC-1115</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -5469,17 +5469,17 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Password redaction</t>
+          <t>Auth after setup — test-connection</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision and check response</t>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>No password in response body</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F172" s="4" t="n"/>
@@ -5490,7 +5490,7 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>TC-1118</t>
+          <t>TC-1116</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
@@ -5500,17 +5500,17 @@
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Re-provision blocked</t>
+          <t>Auth after setup — provision</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>409, already provisioned</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F173" s="4" t="n"/>
@@ -5521,7 +5521,7 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>TC-1119</t>
+          <t>TC-1117</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -5531,17 +5531,17 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision (admin)</t>
+          <t>Password redaction</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+          <t>POST /setup/database/provision and check response</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>No password in response body</t>
         </is>
       </c>
       <c r="F174" s="4" t="n"/>
@@ -5552,7 +5552,7 @@
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>TC-1120</t>
+          <t>TC-1118</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -5562,17 +5562,17 @@
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Force rejected unauthenticated</t>
+          <t>Re-provision blocked</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
         </is>
       </c>
       <c r="E175" s="4" t="inlineStr">
         <is>
-          <t>403, force requires admin</t>
+          <t>409, already provisioned</t>
         </is>
       </c>
       <c r="F175" s="4" t="n"/>
@@ -5583,7 +5583,7 @@
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>TC-1121</t>
+          <t>TC-1119</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -5593,17 +5593,17 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Force re-provision (admin)</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F176" s="4" t="n"/>
@@ -5614,7 +5614,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>TC-1122</t>
+          <t>TC-1120</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -5624,17 +5624,17 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Force rejected unauthenticated</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>403, force requires admin</t>
         </is>
       </c>
       <c r="F177" s="4" t="n"/>
@@ -5645,7 +5645,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>TC-1123</t>
+          <t>TC-1121</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -5655,17 +5655,17 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — provision state unknown</t>
+          <t>Fail-closed — DB unreachable, no JWT</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>503, database unavailable message</t>
         </is>
       </c>
       <c r="F178" s="4" t="n"/>
@@ -5676,7 +5676,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>TC-1124</t>
+          <t>TC-1122</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -5686,17 +5686,17 @@
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Force bypasses state check</t>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>Proceeds to provisioning (no 503 from state check)</t>
+          <t>Request proceeds (not blocked by 503)</t>
         </is>
       </c>
       <c r="F179" s="4" t="n"/>
@@ -5707,7 +5707,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>TC-1125</t>
+          <t>TC-1123</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -5717,17 +5717,17 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>Unmigrated DB treated as initial setup</t>
+          <t>Fail-closed — provision state unknown</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>200, request allowed (not 503)</t>
+          <t>503, cannot determine provisioning state</t>
         </is>
       </c>
       <c r="F180" s="4" t="n"/>
@@ -5738,7 +5738,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>TC-1126</t>
+          <t>TC-1124</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -5748,17 +5748,17 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Fresh install — DB/role missing</t>
+          <t>Force bypasses state check</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>200, provisioning proceeds (not 503)</t>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
         </is>
       </c>
       <c r="F181" s="4" t="n"/>
@@ -5769,7 +5769,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>TC-1127</t>
+          <t>TC-1125</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -5779,17 +5779,17 @@
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — OperationalError on reachable DB</t>
+          <t>Unmigrated DB treated as initial setup</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>200, request allowed (not 503)</t>
         </is>
       </c>
       <c r="F182" s="4" t="n"/>
@@ -5800,7 +5800,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>TC-1128</t>
+          <t>TC-1126</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -5810,17 +5810,17 @@
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — unexpected error</t>
+          <t>Fresh install — DB/role missing</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
         </is>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>200, provisioning proceeds (not 503)</t>
         </is>
       </c>
       <c r="F183" s="4" t="n"/>
@@ -5831,7 +5831,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>TC-1129</t>
+          <t>TC-1127</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -5841,17 +5841,17 @@
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>Provision — migration failure</t>
+          <t>Fail-closed — OperationalError on reachable DB</t>
         </is>
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+          <t>503, does NOT grant unauthenticated access</t>
         </is>
       </c>
       <c r="F184" s="4" t="n"/>
@@ -5862,7 +5862,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>TC-1130</t>
+          <t>TC-1128</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -5872,17 +5872,17 @@
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Provision — .env write failure</t>
+          <t>Fail-closed — unexpected error</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>500, "failed to persist" message; engine not swapped</t>
+          <t>503, does NOT grant unauthenticated access</t>
         </is>
       </c>
       <c r="F185" s="4" t="n"/>
@@ -5893,7 +5893,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>TC-1131</t>
+          <t>TC-1129</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -5903,17 +5903,17 @@
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Provision — engine reinit failure</t>
+          <t>Provision — migration failure</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>500, "engine could not be switched" message; .env already written</t>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
         </is>
       </c>
       <c r="F186" s="4" t="n"/>
@@ -5921,14 +5921,76 @@
       <c r="H186" s="4" t="n"/>
       <c r="I186" s="4" t="n"/>
     </row>
+    <row r="187">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>TC-1130</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>Provision — .env write failure</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+        </is>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>500, "failed to persist" message; engine not swapped</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="n"/>
+      <c r="G187" s="4" t="n"/>
+      <c r="H187" s="4" t="n"/>
+      <c r="I187" s="4" t="n"/>
+    </row>
     <row r="188">
-      <c r="A188" s="5" t="inlineStr">
+      <c r="A188" s="4" t="inlineStr">
+        <is>
+          <t>TC-1131</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C188" s="4" t="inlineStr">
+        <is>
+          <t>Provision — engine reinit failure</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+        </is>
+      </c>
+      <c r="E188" s="4" t="inlineStr">
+        <is>
+          <t>500, "engine could not be switched" message; .env already written</t>
+        </is>
+      </c>
+      <c r="F188" s="4" t="n"/>
+      <c r="G188" s="4" t="n"/>
+      <c r="H188" s="4" t="n"/>
+      <c r="I188" s="4" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B188" s="5" t="n">
-        <v>171</v>
+      <c r="B190" s="5" t="n">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hub & Port Identification Enrichment
</commit_message>
<xml_diff>
--- a/documents/testing/ecube-qa-test-cases.xlsx
+++ b/documents/testing/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I190"/>
+  <dimension ref="A1:I208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2626,12 +2626,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>§12.5 USB Hardware</t>
+          <t>§12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C77" s="3" t="n"/>
@@ -2645,27 +2645,27 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>TC-501</t>
+          <t>TC-441</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Hot-plug detection</t>
+          <t>List hubs — admin</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>Plug in a USB drive, wait 30 seconds</t>
+          <t>GET /admin/hubs with admin token</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>GET /drives shows the new drive (in EMPTY state if port is disabled, or AVAILABLE if port is enabled)</t>
+          <t>200, array of hub objects with vendor_id, product_id, location_hint</t>
         </is>
       </c>
       <c r="F78" s="4" t="n"/>
@@ -2676,27 +2676,27 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>TC-502</t>
+          <t>TC-442</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>USB topology</t>
+          <t>List hubs — manager</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>GET /introspection/usb/topology</t>
+          <t>GET /admin/hubs with manager token</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>Shows real hub serial numbers, port numbers, connected devices</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F79" s="4" t="n"/>
@@ -2707,27 +2707,27 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>TC-503</t>
+          <t>TC-443</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Physical eject</t>
+          <t>List hubs — processor denied</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>Initialize drive → prepare-eject → physically remove</t>
+          <t>GET /admin/hubs with processor token</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F80" s="4" t="n"/>
@@ -2738,27 +2738,27 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>TC-504</t>
+          <t>TC-444</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Re-plug same drive</t>
+          <t>List hubs — unauthenticated</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>Remove and re-insert the same drive</t>
+          <t>GET /admin/hubs without token</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F81" s="4" t="n"/>
@@ -2769,27 +2769,27 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>TC-505</t>
+          <t>TC-445</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Multiple drives</t>
+          <t>Set hub location hint</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>Plug in 2+ drives simultaneously</t>
+          <t>PATCH /admin/hubs/{id} with {"location_hint": "back-left rack"}</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>All drives appear in /drives; each can be initialized to different projects</t>
+          <t>200, hub returned with location_hint: "back-left rack"</t>
         </is>
       </c>
       <c r="F82" s="4" t="n"/>
@@ -2800,27 +2800,27 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>TC-506</t>
+          <t>TC-446</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Sync + unmount</t>
+          <t>Set hub location hint — manager</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>Initialize drive, create/start a job, then prepare-eject</t>
+          <t>PATCH /admin/hubs/{id} with manager token</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F83" s="4" t="n"/>
@@ -2831,27 +2831,27 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>TC-507</t>
+          <t>TC-447</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>12.5 USB Hardware</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Disabled port blocks AVAILABLE</t>
+          <t>Set hub location hint — processor denied</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>Disable a port, plug in a drive to that port, run discovery</t>
+          <t>PATCH /admin/hubs/{id} with processor token</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Drive appears in EMPTY state; enable port + refresh → drive transitions to AVAILABLE</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F84" s="4" t="n"/>
@@ -2860,48 +2860,60 @@
       <c r="I84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>§12.6 End-to-End Copy</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>12.6 End-to-End Copy</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="n"/>
-      <c r="D85" s="3" t="n"/>
-      <c r="E85" s="3" t="n"/>
-      <c r="F85" s="3" t="n"/>
-      <c r="G85" s="3" t="n"/>
-      <c r="H85" s="3" t="n"/>
-      <c r="I85" s="3" t="n"/>
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>TC-448</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>12.4.4 Hub/Port Enrichment</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Set hub location hint — not found</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/hubs/99999</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>404, NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="n"/>
+      <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>TC-601</t>
+          <t>TC-449</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>12.6 End-to-End Copy</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Full E2E workflow</t>
+          <t>HUB_LABEL_UPDATED audit log</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>Setup test files → add mount → discover drive → initialize → create job → start → poll → verify → manifest → eject → verify on another machine</t>
+          <t>GET /audit?action=HUB_LABEL_UPDATED after setting a hub label</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>All steps succeed; checksums match; audit trail shows complete chain</t>
+          <t>Audit entry with hub_id, system_identifier, field, old_value, new_value, path</t>
         </is>
       </c>
       <c r="F86" s="4" t="n"/>
@@ -2910,44 +2922,60 @@
       <c r="I86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>§12.7 Error Handling</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>12.7 Error Handling</t>
-        </is>
-      </c>
-      <c r="C87" s="3" t="n"/>
-      <c r="D87" s="3" t="n"/>
-      <c r="E87" s="3" t="n"/>
-      <c r="F87" s="3" t="n"/>
-      <c r="G87" s="3" t="n"/>
-      <c r="H87" s="3" t="n"/>
-      <c r="I87" s="3" t="n"/>
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>TC-450</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>12.4.4 Hub/Port Enrichment</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Set port friendly label</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/ports/{id}/label with {"friendly_label": "Bay 3"}</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>200, port returned with friendly_label: "Bay 3"</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="n"/>
+      <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>TC-701</t>
+          <t>TC-451</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>GET /jobs/99999</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr"/>
+          <t>Set port friendly label — manager</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/ports/{id}/label with manager token</t>
+        </is>
+      </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F88" s="4" t="n"/>
@@ -2958,23 +2986,27 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>TC-702</t>
+          <t>TC-452</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>DELETE /mounts/99999</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr"/>
+          <t>Set port friendly label — processor denied</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/ports/{id}/label with processor token</t>
+        </is>
+      </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F89" s="4" t="n"/>
@@ -2985,23 +3017,27 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>TC-703</t>
+          <t>TC-453</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Start an already-running job</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr"/>
+          <t>Set port friendly label — not found</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>PATCH /admin/ports/{id}/label for non-existent port</t>
+        </is>
+      </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>409, CONFLICT</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F90" s="4" t="n"/>
@@ -3012,23 +3048,27 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>TC-704</t>
+          <t>TC-454</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>All error responses</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr"/>
+          <t>PORT_LABEL_UPDATED audit log</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>GET /audit?action=PORT_LABEL_UPDATED after setting a port label</t>
+        </is>
+      </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>JSON body includes code, message, and trace_id</t>
+          <t>Audit entry with port_id, system_path, field, old_value, new_value, path</t>
         </is>
       </c>
       <c r="F91" s="4" t="n"/>
@@ -3039,23 +3079,27 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>TC-705</t>
+          <t>TC-455</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/999/format with {"filesystem_type": "ext4"}</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr"/>
+          <t>Port listing includes enriched fields</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>GET /admin/ports after discovery</t>
+        </is>
+      </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>Port objects include vendor_id, product_id, speed fields</t>
         </is>
       </c>
       <c r="F92" s="4" t="n"/>
@@ -3066,23 +3110,27 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>TC-706</t>
+          <t>TC-456</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr"/>
+          <t>Labels survive discovery resync</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Set hub location_hint and port friendly_label, then POST /drives/refresh</t>
+        </is>
+      </c>
       <c r="E93" s="4" t="inlineStr">
         <is>
-          <t>422, validation error</t>
+          <t>Labels remain unchanged after resync</t>
         </is>
       </c>
       <c r="F93" s="4" t="n"/>
@@ -3093,23 +3141,27 @@
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>TC-707</t>
+          <t>TC-457</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>12.7 Error Handling</t>
+          <t>12.4.4 Hub/Port Enrichment</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>POST /drives/{id}/format with empty body</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr"/>
+          <t>Discovery populates vendor/product IDs</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Run POST /drives/refresh with USB hardware connected</t>
+        </is>
+      </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Hub and port records show vendor_id and product_id from sysfs</t>
         </is>
       </c>
       <c r="F94" s="4" t="n"/>
@@ -3120,12 +3172,12 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>§12.8 User Role Mgmt</t>
+          <t>§12.5 USB Hardware</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C95" s="3" t="n"/>
@@ -3139,27 +3191,27 @@
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>TC-801</t>
+          <t>TC-501</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>List users (empty)</t>
+          <t>Hot-plug detection</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>GET /users with admin token (no roles assigned yet)</t>
+          <t>Plug in a USB drive, wait 30 seconds</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>200, {"users": []}</t>
+          <t>GET /drives shows the new drive (in EMPTY state if port is disabled, or AVAILABLE if port is enabled)</t>
         </is>
       </c>
       <c r="F96" s="4" t="n"/>
@@ -3170,27 +3222,27 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>TC-802</t>
+          <t>TC-502</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Assign roles</t>
+          <t>USB topology</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["processor", "auditor"]}</t>
+          <t>GET /introspection/usb/topology</t>
         </is>
       </c>
       <c r="E97" s="4" t="inlineStr">
         <is>
-          <t>200, returns username and sorted roles</t>
+          <t>Shows real hub serial numbers, port numbers, connected devices</t>
         </is>
       </c>
       <c r="F97" s="4" t="n"/>
@@ -3201,27 +3253,27 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>TC-803</t>
+          <t>TC-503</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Get roles</t>
+          <t>Physical eject</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>GET /users/qa-processor/roles after assignment</t>
+          <t>Initialize drive → prepare-eject → physically remove</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
+          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
         </is>
       </c>
       <c r="F98" s="4" t="n"/>
@@ -3232,27 +3284,27 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>TC-804</t>
+          <t>TC-504</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>List users after assignment</t>
+          <t>Re-plug same drive</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>GET /users after assigning roles</t>
+          <t>Remove and re-insert the same drive</t>
         </is>
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>200, user appears in list with correct roles</t>
+          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
         </is>
       </c>
       <c r="F99" s="4" t="n"/>
@@ -3263,27 +3315,27 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>TC-805</t>
+          <t>TC-505</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Replace roles</t>
+          <t>Multiple drives</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["manager"]}</t>
+          <t>Plug in 2+ drives simultaneously</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>200, only ["manager"] returned; old roles removed</t>
+          <t>All drives appear in /drives; each can be initialized to different projects</t>
         </is>
       </c>
       <c r="F100" s="4" t="n"/>
@@ -3294,27 +3346,27 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>TC-806</t>
+          <t>TC-506</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Deduplicate roles</t>
+          <t>Sync + unmount</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
+          <t>Initialize drive, create/start a job, then prepare-eject</t>
         </is>
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>200, deduplicated to ["admin", "processor"]</t>
+          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
         </is>
       </c>
       <c r="F101" s="4" t="n"/>
@@ -3325,27 +3377,27 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>TC-807</t>
+          <t>TC-507</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.5 USB Hardware</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Invalid role name</t>
+          <t>Disabled port blocks AVAILABLE</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
+          <t>Disable a port, plug in a drive to that port, run discovery</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>422, error message mentions superuser</t>
+          <t>Drive appears in EMPTY state; enable port + refresh → drive transitions to AVAILABLE</t>
         </is>
       </c>
       <c r="F102" s="4" t="n"/>
@@ -3354,60 +3406,48 @@
       <c r="I102" s="4" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr">
-        <is>
-          <t>TC-808</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>Empty role list</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="inlineStr">
-        <is>
-          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
-        </is>
-      </c>
-      <c r="E103" s="4" t="inlineStr">
-        <is>
-          <t>422, at least one role required</t>
-        </is>
-      </c>
-      <c r="F103" s="4" t="n"/>
-      <c r="G103" s="4" t="n"/>
-      <c r="H103" s="4" t="n"/>
-      <c r="I103" s="4" t="n"/>
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>§12.6 End-to-End Copy</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>12.6 End-to-End Copy</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="n"/>
+      <c r="D103" s="3" t="n"/>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="3" t="n"/>
+      <c r="G103" s="3" t="n"/>
+      <c r="H103" s="3" t="n"/>
+      <c r="I103" s="3" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>TC-809</t>
+          <t>TC-601</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.6 End-to-End Copy</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Remove roles</t>
+          <t>Full E2E workflow</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>DELETE /users/qa-processor/roles</t>
+          <t>Setup test files → add mount → discover drive → initialize → create job → start → poll → verify → manifest → eject → verify on another machine</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "qa-processor", "roles": []}</t>
+          <t>All steps succeed; checksums match; audit trail shows complete chain</t>
         </is>
       </c>
       <c r="F104" s="4" t="n"/>
@@ -3416,60 +3456,44 @@
       <c r="I104" s="4" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="4" t="inlineStr">
-        <is>
-          <t>TC-810</t>
-        </is>
-      </c>
-      <c r="B105" s="4" t="inlineStr">
-        <is>
-          <t>12.8 User Role Mgmt</t>
-        </is>
-      </c>
-      <c r="C105" s="4" t="inlineStr">
-        <is>
-          <t>Get roles after removal</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>GET /users/qa-processor/roles after DELETE</t>
-        </is>
-      </c>
-      <c r="E105" s="4" t="inlineStr">
-        <is>
-          <t>200, {"roles": []}</t>
-        </is>
-      </c>
-      <c r="F105" s="4" t="n"/>
-      <c r="G105" s="4" t="n"/>
-      <c r="H105" s="4" t="n"/>
-      <c r="I105" s="4" t="n"/>
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>§12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="n"/>
+      <c r="D105" s="3" t="n"/>
+      <c r="E105" s="3" t="n"/>
+      <c r="F105" s="3" t="n"/>
+      <c r="G105" s="3" t="n"/>
+      <c r="H105" s="3" t="n"/>
+      <c r="I105" s="3" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>TC-811</t>
+          <t>TC-701</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Get roles for unknown user</t>
-        </is>
-      </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>GET /users/nonexistent/roles</t>
-        </is>
-      </c>
+          <t>GET /jobs/99999</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr"/>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>200, {"username": "nonexistent", "roles": []}</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F106" s="4" t="n"/>
@@ -3480,27 +3504,23 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>TC-812</t>
+          <t>TC-702</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot list users</t>
-        </is>
-      </c>
-      <c r="D107" s="4" t="inlineStr">
-        <is>
-          <t>GET /users with processor token</t>
-        </is>
-      </c>
+          <t>DELETE /mounts/99999</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr"/>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F107" s="4" t="n"/>
@@ -3511,27 +3531,23 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>TC-813</t>
+          <t>TC-703</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot set roles</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="inlineStr">
-        <is>
-          <t>PUT /users/x/roles with processor token</t>
-        </is>
-      </c>
+          <t>Start an already-running job</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr"/>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>409, CONFLICT</t>
         </is>
       </c>
       <c r="F108" s="4" t="n"/>
@@ -3542,27 +3558,23 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>TC-814</t>
+          <t>TC-704</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot delete roles</t>
-        </is>
-      </c>
-      <c r="D109" s="4" t="inlineStr">
-        <is>
-          <t>DELETE /users/x/roles with processor token</t>
-        </is>
-      </c>
+          <t>All error responses</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr"/>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>JSON body includes code, message, and trace_id</t>
         </is>
       </c>
       <c r="F109" s="4" t="n"/>
@@ -3573,27 +3585,23 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>TC-815</t>
+          <t>TC-705</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Unauthenticated access</t>
-        </is>
-      </c>
-      <c r="D110" s="4" t="inlineStr">
-        <is>
-          <t>GET /users without Authorization header</t>
-        </is>
-      </c>
+          <t>POST /drives/999/format with {"filesystem_type": "ext4"}</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr"/>
       <c r="E110" s="4" t="inlineStr">
         <is>
-          <t>401, UNAUTHORIZED</t>
+          <t>404, NOT_FOUND</t>
         </is>
       </c>
       <c r="F110" s="4" t="n"/>
@@ -3604,27 +3612,23 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>TC-816</t>
+          <t>TC-706</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>ROLE_ASSIGNED audit log</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>GET /audit?action=ROLE_ASSIGNED after assigning roles</t>
-        </is>
-      </c>
+          <t>POST /drives/{id}/format with {"filesystem_type": "ntfs"}</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr"/>
       <c r="E111" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor, target user, and roles</t>
+          <t>422, validation error</t>
         </is>
       </c>
       <c r="F111" s="4" t="n"/>
@@ -3635,27 +3639,23 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>TC-817</t>
+          <t>TC-707</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>12.8 User Role Mgmt</t>
+          <t>12.7 Error Handling</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>ROLE_REMOVED audit log</t>
-        </is>
-      </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>GET /audit?action=ROLE_REMOVED after removing roles</t>
-        </is>
-      </c>
+          <t>POST /drives/{id}/format with empty body</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr"/>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and target user</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F112" s="4" t="n"/>
@@ -3664,40 +3664,28 @@
       <c r="I112" s="4" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>TC-818</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>§12.8 User Role Mgmt</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>DB roles override groups</t>
-        </is>
-      </c>
-      <c r="D113" s="4" t="inlineStr">
-        <is>
-          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="n"/>
-      <c r="G113" s="4" t="n"/>
-      <c r="H113" s="4" t="n"/>
-      <c r="I113" s="4" t="n"/>
+      <c r="C113" s="3" t="n"/>
+      <c r="D113" s="3" t="n"/>
+      <c r="E113" s="3" t="n"/>
+      <c r="F113" s="3" t="n"/>
+      <c r="G113" s="3" t="n"/>
+      <c r="H113" s="3" t="n"/>
+      <c r="I113" s="3" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>TC-819</t>
+          <t>TC-801</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
@@ -3707,17 +3695,17 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>Fallback to group roles</t>
+          <t>List users (empty)</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
+          <t>GET /users with admin token (no roles assigned yet)</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>JWT roles falls back to OS group mapping (["processor"])</t>
+          <t>200, {"users": []}</t>
         </is>
       </c>
       <c r="F114" s="4" t="n"/>
@@ -3726,48 +3714,60 @@
       <c r="I114" s="4" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>§12.9 OS User &amp; Group Mgmt</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
-        <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
-        </is>
-      </c>
-      <c r="C115" s="3" t="n"/>
-      <c r="D115" s="3" t="n"/>
-      <c r="E115" s="3" t="n"/>
-      <c r="F115" s="3" t="n"/>
-      <c r="G115" s="3" t="n"/>
-      <c r="H115" s="3" t="n"/>
-      <c r="I115" s="3" t="n"/>
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>TC-802</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>12.8 User Role Mgmt</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>Assign roles</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>PUT /users/qa-processor/roles with {"roles": ["processor", "auditor"]}</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>200, returns username and sorted roles</t>
+        </is>
+      </c>
+      <c r="F115" s="4" t="n"/>
+      <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
+      <c r="I115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>TC-901</t>
+          <t>TC-803</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>Create group</t>
+          <t>Get roles</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
+          <t>GET /users/qa-processor/roles after assignment</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>201, returns name, gid, members</t>
+          <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
         </is>
       </c>
       <c r="F116" s="4" t="n"/>
@@ -3778,27 +3778,27 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>TC-902</t>
+          <t>TC-804</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Create group without prefix</t>
+          <t>List users after assignment</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-groups with {"name": "testers"}</t>
+          <t>GET /users after assigning roles</t>
         </is>
       </c>
       <c r="E117" s="4" t="inlineStr">
         <is>
-          <t>422, group name must start with ecube-</t>
+          <t>200, user appears in list with correct roles</t>
         </is>
       </c>
       <c r="F117" s="4" t="n"/>
@@ -3809,27 +3809,27 @@
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>TC-903</t>
+          <t>TC-805</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>List groups</t>
+          <t>Replace roles</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-groups</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["manager"]}</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>200, only ecube-* groups listed</t>
+          <t>200, only ["manager"] returned; old roles removed</t>
         </is>
       </c>
       <c r="F118" s="4" t="n"/>
@@ -3840,27 +3840,27 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>TC-904</t>
+          <t>TC-806</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>Delete group</t>
+          <t>Deduplicate roles</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-groups/ecube-testers</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
         </is>
       </c>
       <c r="E119" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, deduplicated to ["admin", "processor"]</t>
         </is>
       </c>
       <c r="F119" s="4" t="n"/>
@@ -3871,27 +3871,27 @@
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
         <is>
-          <t>TC-905</t>
+          <t>TC-807</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>Delete group without prefix</t>
+          <t>Invalid role name</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-groups/somegroup</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>422, group name must start with ecube-</t>
+          <t>422, error message mentions superuser</t>
         </is>
       </c>
       <c r="F120" s="4" t="n"/>
@@ -3902,27 +3902,27 @@
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
         <is>
-          <t>TC-906</t>
+          <t>TC-808</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>Create user</t>
+          <t>Empty role list</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with username, password, groups, roles</t>
+          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
         </is>
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>201, returns username, uid, gid, home, shell, groups</t>
+          <t>422, at least one role required</t>
         </is>
       </c>
       <c r="F121" s="4" t="n"/>
@@ -3933,27 +3933,27 @@
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
         <is>
-          <t>TC-907</t>
+          <t>TC-809</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>Create user — duplicate</t>
+          <t>Remove roles</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with existing username</t>
+          <t>DELETE /users/qa-processor/roles</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200, {"username": "qa-processor", "roles": []}</t>
         </is>
       </c>
       <c r="F122" s="4" t="n"/>
@@ -3964,27 +3964,27 @@
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
         <is>
-          <t>TC-908</t>
+          <t>TC-810</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>Create user — reserved name</t>
+          <t>Get roles after removal</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"username": "root", ...}</t>
+          <t>GET /users/qa-processor/roles after DELETE</t>
         </is>
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>422, reserved username</t>
+          <t>200, {"roles": []}</t>
         </is>
       </c>
       <c r="F123" s="4" t="n"/>
@@ -3995,27 +3995,27 @@
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
         <is>
-          <t>TC-909</t>
+          <t>TC-811</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>Create user — empty password</t>
+          <t>Get roles for unknown user</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with {"password": "", ...}</t>
+          <t>GET /users/nonexistent/roles</t>
         </is>
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, {"username": "nonexistent", "roles": []}</t>
         </is>
       </c>
       <c r="F124" s="4" t="n"/>
@@ -4026,27 +4026,27 @@
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
         <is>
-          <t>TC-910</t>
+          <t>TC-812</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with newline</t>
+          <t>Processor cannot list users</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing \n</t>
+          <t>GET /users with processor token</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F125" s="4" t="n"/>
@@ -4057,27 +4057,27 @@
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
         <is>
-          <t>TC-911</t>
+          <t>TC-813</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>Create user — password with colon</t>
+          <t>Processor cannot set roles</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with password containing :</t>
+          <t>PUT /users/x/roles with processor token</t>
         </is>
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F126" s="4" t="n"/>
@@ -4088,27 +4088,27 @@
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
         <is>
-          <t>TC-912</t>
+          <t>TC-814</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>Create user — invalid group</t>
+          <t>Processor cannot delete roles</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with non-existent group in groups list</t>
+          <t>DELETE /users/x/roles with processor token</t>
         </is>
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>422, group does not exist</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F127" s="4" t="n"/>
@@ -4119,27 +4119,27 @@
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
         <is>
-          <t>TC-913</t>
+          <t>TC-815</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>Create user — no ecube-* group</t>
+          <t>Unauthenticated access</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
+          <t>GET /users without Authorization header</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>422, at least one ecube-* group required</t>
+          <t>401, UNAUTHORIZED</t>
         </is>
       </c>
       <c r="F128" s="4" t="n"/>
@@ -4150,27 +4150,27 @@
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
         <is>
-          <t>TC-914</t>
+          <t>TC-816</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>List users</t>
+          <t>ROLE_ASSIGNED audit log</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users</t>
+          <t>GET /audit?action=ROLE_ASSIGNED after assigning roles</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>200, only users in ecube-* groups listed</t>
+          <t>Audit entry with actor, target user, and roles</t>
         </is>
       </c>
       <c r="F129" s="4" t="n"/>
@@ -4181,27 +4181,27 @@
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
         <is>
-          <t>TC-915</t>
+          <t>TC-817</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Reset password</t>
+          <t>ROLE_REMOVED audit log</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+          <t>GET /audit?action=ROLE_REMOVED after removing roles</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>Audit entry with actor and target user</t>
         </is>
       </c>
       <c r="F130" s="4" t="n"/>
@@ -4212,27 +4212,27 @@
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
         <is>
-          <t>TC-916</t>
+          <t>TC-818</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Reset password — non-ECUBE user</t>
+          <t>DB roles override groups</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/postgres/password</t>
+          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
         </is>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
         </is>
       </c>
       <c r="F131" s="4" t="n"/>
@@ -4243,27 +4243,27 @@
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
         <is>
-          <t>TC-917</t>
+          <t>TC-819</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>12.9 OS User &amp; Group Mgmt</t>
+          <t>12.8 User Role Mgmt</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>Replace groups</t>
+          <t>Fallback to group roles</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
+          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
         </is>
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list; non-ecube-* groups preserved</t>
+          <t>JWT roles falls back to OS group mapping (["processor"])</t>
         </is>
       </c>
       <c r="F132" s="4" t="n"/>
@@ -4272,40 +4272,28 @@
       <c r="I132" s="4" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="4" t="inlineStr">
-        <is>
-          <t>TC-918</t>
-        </is>
-      </c>
-      <c r="B133" s="4" t="inlineStr">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>§12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C133" s="4" t="inlineStr">
-        <is>
-          <t>Replace groups — empty list</t>
-        </is>
-      </c>
-      <c r="D133" s="4" t="inlineStr">
-        <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
-        </is>
-      </c>
-      <c r="E133" s="4" t="inlineStr">
-        <is>
-          <t>422, at least one ecube-* group required</t>
-        </is>
-      </c>
-      <c r="F133" s="4" t="n"/>
-      <c r="G133" s="4" t="n"/>
-      <c r="H133" s="4" t="n"/>
-      <c r="I133" s="4" t="n"/>
+      <c r="C133" s="3" t="n"/>
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
+      <c r="F133" s="3" t="n"/>
+      <c r="G133" s="3" t="n"/>
+      <c r="H133" s="3" t="n"/>
+      <c r="I133" s="3" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
         <is>
-          <t>TC-919</t>
+          <t>TC-901</t>
         </is>
       </c>
       <c r="B134" s="4" t="inlineStr">
@@ -4315,17 +4303,17 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>Replace groups — non-ecube name</t>
+          <t>Create group</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
+          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>422, group does not start with ecube-</t>
+          <t>201, returns name, gid, members</t>
         </is>
       </c>
       <c r="F134" s="4" t="n"/>
@@ -4336,7 +4324,7 @@
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
         <is>
-          <t>TC-920</t>
+          <t>TC-902</t>
         </is>
       </c>
       <c r="B135" s="4" t="inlineStr">
@@ -4346,17 +4334,17 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>Append groups</t>
+          <t>Create group without prefix</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+          <t>POST /admin/os-groups with {"name": "testers"}</t>
         </is>
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
+          <t>422, group name must start with ecube-</t>
         </is>
       </c>
       <c r="F135" s="4" t="n"/>
@@ -4367,7 +4355,7 @@
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
         <is>
-          <t>TC-921</t>
+          <t>TC-903</t>
         </is>
       </c>
       <c r="B136" s="4" t="inlineStr">
@@ -4377,17 +4365,17 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>Modify groups — non-ECUBE user</t>
+          <t>List groups</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/www-data/groups</t>
+          <t>GET /admin/os-groups</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200, only ecube-* groups listed</t>
         </is>
       </c>
       <c r="F136" s="4" t="n"/>
@@ -4398,7 +4386,7 @@
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
         <is>
-          <t>TC-922</t>
+          <t>TC-904</t>
         </is>
       </c>
       <c r="B137" s="4" t="inlineStr">
@@ -4408,17 +4396,17 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>Delete user</t>
+          <t>Delete group</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/{username}</t>
+          <t>DELETE /admin/os-groups/ecube-testers</t>
         </is>
       </c>
       <c r="E137" s="4" t="inlineStr">
         <is>
-          <t>200, user and DB roles removed</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F137" s="4" t="n"/>
@@ -4429,7 +4417,7 @@
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
         <is>
-          <t>TC-923</t>
+          <t>TC-905</t>
         </is>
       </c>
       <c r="B138" s="4" t="inlineStr">
@@ -4439,17 +4427,17 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>Delete user — non-ECUBE user</t>
+          <t>Delete group without prefix</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/daemon</t>
+          <t>DELETE /admin/os-groups/somegroup</t>
         </is>
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>422, group name must start with ecube-</t>
         </is>
       </c>
       <c r="F138" s="4" t="n"/>
@@ -4460,7 +4448,7 @@
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
         <is>
-          <t>TC-924</t>
+          <t>TC-906</t>
         </is>
       </c>
       <c r="B139" s="4" t="inlineStr">
@@ -4470,17 +4458,17 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>Delete user — not found</t>
+          <t>Create user</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/nonexistent</t>
+          <t>POST /admin/os-users with username, password, groups, roles</t>
         </is>
       </c>
       <c r="E139" s="4" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>201, returns username, uid, gid, home, shell, groups</t>
         </is>
       </c>
       <c r="F139" s="4" t="n"/>
@@ -4491,7 +4479,7 @@
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
         <is>
-          <t>TC-925</t>
+          <t>TC-907</t>
         </is>
       </c>
       <c r="B140" s="4" t="inlineStr">
@@ -4501,17 +4489,17 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>Processor cannot access OS endpoints</t>
+          <t>Create user — duplicate</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>GET /admin/os-users with processor token</t>
+          <t>POST /admin/os-users with existing username</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F140" s="4" t="n"/>
@@ -4522,7 +4510,7 @@
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
         <is>
-          <t>TC-926</t>
+          <t>TC-908</t>
         </is>
       </c>
       <c r="B141" s="4" t="inlineStr">
@@ -4532,17 +4520,17 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>Non-local mode returns 404</t>
+          <t>Create user — reserved name</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+          <t>POST /admin/os-users with {"username": "root", ...}</t>
         </is>
       </c>
       <c r="E141" s="4" t="inlineStr">
         <is>
-          <t>404, Not Found</t>
+          <t>422, reserved username</t>
         </is>
       </c>
       <c r="F141" s="4" t="n"/>
@@ -4553,7 +4541,7 @@
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
         <is>
-          <t>TC-927</t>
+          <t>TC-909</t>
         </is>
       </c>
       <c r="B142" s="4" t="inlineStr">
@@ -4563,17 +4551,17 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_CREATED audit log</t>
+          <t>Create user — empty password</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+          <t>POST /admin/os-users with {"password": "", ...}</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F142" s="4" t="n"/>
@@ -4584,7 +4572,7 @@
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
         <is>
-          <t>TC-928</t>
+          <t>TC-910</t>
         </is>
       </c>
       <c r="B143" s="4" t="inlineStr">
@@ -4594,17 +4582,17 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>OS_USER_DELETED audit log</t>
+          <t>Create user — password with newline</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+          <t>POST /admin/os-users with password containing \n</t>
         </is>
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F143" s="4" t="n"/>
@@ -4615,7 +4603,7 @@
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
         <is>
-          <t>TC-929</t>
+          <t>TC-911</t>
         </is>
       </c>
       <c r="B144" s="4" t="inlineStr">
@@ -4625,17 +4613,17 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>OS_PASSWORD_RESET audit log</t>
+          <t>Create user — password with colon</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+          <t>POST /admin/os-users with password containing :</t>
         </is>
       </c>
       <c r="E144" s="4" t="inlineStr">
         <is>
-          <t>Audit entry (no password in details)</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F144" s="4" t="n"/>
@@ -4646,7 +4634,7 @@
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
         <is>
-          <t>TC-930</t>
+          <t>TC-912</t>
         </is>
       </c>
       <c r="B145" s="4" t="inlineStr">
@@ -4656,17 +4644,17 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_CREATED audit log</t>
+          <t>Create user — invalid group</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+          <t>POST /admin/os-users with non-existent group in groups list</t>
         </is>
       </c>
       <c r="E145" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>422, group does not exist</t>
         </is>
       </c>
       <c r="F145" s="4" t="n"/>
@@ -4677,7 +4665,7 @@
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
         <is>
-          <t>TC-931</t>
+          <t>TC-913</t>
         </is>
       </c>
       <c r="B146" s="4" t="inlineStr">
@@ -4687,17 +4675,17 @@
       </c>
       <c r="C146" s="4" t="inlineStr">
         <is>
-          <t>OS_GROUP_DELETED audit log</t>
+          <t>Create user — no ecube-* group</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F146" s="4" t="n"/>
@@ -4706,48 +4694,60 @@
       <c r="I146" s="4" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="inlineStr">
-        <is>
-          <t>§12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B147" s="2" t="inlineStr">
-        <is>
-          <t>12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C147" s="3" t="n"/>
-      <c r="D147" s="3" t="n"/>
-      <c r="E147" s="3" t="n"/>
-      <c r="F147" s="3" t="n"/>
-      <c r="G147" s="3" t="n"/>
-      <c r="H147" s="3" t="n"/>
-      <c r="I147" s="3" t="n"/>
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>TC-914</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>List users</t>
+        </is>
+      </c>
+      <c r="D147" s="4" t="inlineStr">
+        <is>
+          <t>GET /admin/os-users</t>
+        </is>
+      </c>
+      <c r="E147" s="4" t="inlineStr">
+        <is>
+          <t>200, only users in ecube-* groups listed</t>
+        </is>
+      </c>
+      <c r="F147" s="4" t="n"/>
+      <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
+      <c r="I147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>TC-1001</t>
+          <t>TC-915</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>Reset password</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
         </is>
       </c>
       <c r="E148" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F148" s="4" t="n"/>
@@ -4758,27 +4758,27 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>TC-1002</t>
+          <t>TC-916</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>Reset password — non-ECUBE user</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with valid username and password</t>
+          <t>PUT /admin/os-users/postgres/password</t>
         </is>
       </c>
       <c r="E149" s="4" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F149" s="4" t="n"/>
@@ -4789,27 +4789,27 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-917</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Replace groups</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, updated group list; non-ecube-* groups preserved</t>
         </is>
       </c>
       <c r="F150" s="4" t="n"/>
@@ -4820,27 +4820,27 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-918</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>Replace groups — empty list</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
         </is>
       </c>
       <c r="E151" s="4" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F151" s="4" t="n"/>
@@ -4851,27 +4851,27 @@
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-919</t>
         </is>
       </c>
       <c r="B152" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C152" s="4" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Replace groups — non-ecube name</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
         </is>
       </c>
       <c r="E152" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>422, group does not start with ecube-</t>
         </is>
       </c>
       <c r="F152" s="4" t="n"/>
@@ -4882,27 +4882,27 @@
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-920</t>
         </is>
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C153" s="4" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Append groups</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
       <c r="E153" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, updated group list</t>
         </is>
       </c>
       <c r="F153" s="4" t="n"/>
@@ -4913,27 +4913,27 @@
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-921</t>
         </is>
       </c>
       <c r="B154" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C154" s="4" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
       <c r="D154" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
       <c r="E154" s="4" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F154" s="4" t="n"/>
@@ -4944,27 +4944,27 @@
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-922</t>
         </is>
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C155" s="4" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Delete user</t>
         </is>
       </c>
       <c r="D155" s="4" t="inlineStr">
         <is>
-          <t>POST /auth/token with the admin credentials from step 2</t>
+          <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
       <c r="E155" s="4" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>200, user and DB roles removed</t>
         </is>
       </c>
       <c r="F155" s="4" t="n"/>
@@ -4975,27 +4975,27 @@
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-923</t>
         </is>
       </c>
       <c r="B156" s="4" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C156" s="4" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F156" s="4" t="n"/>
@@ -5004,48 +5004,60 @@
       <c r="I156" s="4" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="inlineStr">
-        <is>
-          <t>§12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="B157" s="2" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C157" s="3" t="n"/>
-      <c r="D157" s="3" t="n"/>
-      <c r="E157" s="3" t="n"/>
-      <c r="F157" s="3" t="n"/>
-      <c r="G157" s="3" t="n"/>
-      <c r="H157" s="3" t="n"/>
-      <c r="I157" s="3" t="n"/>
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>TC-924</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Delete user — not found</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>DELETE /admin/os-users/nonexistent</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="n"/>
+      <c r="G157" s="4" t="n"/>
+      <c r="H157" s="4" t="n"/>
+      <c r="I157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
         <is>
-          <t>TC-1101</t>
+          <t>TC-925</t>
         </is>
       </c>
       <c r="B158" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C158" s="4" t="inlineStr">
         <is>
-          <t>Test connection — success</t>
+          <t>Processor cannot access OS endpoints</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+          <t>GET /admin/os-users with processor token</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "ok", "server_version": "..."}</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F158" s="4" t="n"/>
@@ -5056,27 +5068,27 @@
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
         <is>
-          <t>TC-1102</t>
+          <t>TC-926</t>
         </is>
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C159" s="4" t="inlineStr">
         <is>
-          <t>Test connection — bad host</t>
+          <t>Non-local mode returns 404</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with unreachable host</t>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>404, Not Found</t>
         </is>
       </c>
       <c r="F159" s="4" t="n"/>
@@ -5087,27 +5099,27 @@
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
         <is>
-          <t>TC-1103</t>
+          <t>TC-927</t>
         </is>
       </c>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C160" s="4" t="inlineStr">
         <is>
-          <t>Test connection — SSRF host</t>
+          <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
         <is>
-          <t>422, invalid host</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F160" s="4" t="n"/>
@@ -5118,27 +5130,27 @@
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
         <is>
-          <t>TC-1104</t>
+          <t>TC-928</t>
         </is>
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C161" s="4" t="inlineStr">
         <is>
-          <t>Test connection — port out of range</t>
+          <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection with "port": 99999</t>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
       <c r="E161" s="4" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F161" s="4" t="n"/>
@@ -5149,27 +5161,27 @@
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
         <is>
-          <t>TC-1105</t>
+          <t>TC-929</t>
         </is>
       </c>
       <c r="B162" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C162" s="4" t="inlineStr">
         <is>
-          <t>Provision — success</t>
+          <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials</t>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>Audit entry (no password in details)</t>
         </is>
       </c>
       <c r="F162" s="4" t="n"/>
@@ -5180,27 +5192,27 @@
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
         <is>
-          <t>TC-1106</t>
+          <t>TC-930</t>
         </is>
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C163" s="4" t="inlineStr">
         <is>
-          <t>Provision — bad admin credentials</t>
+          <t>OS_GROUP_CREATED audit log</t>
         </is>
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with wrong admin password</t>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
         </is>
       </c>
       <c r="E163" s="4" t="inlineStr">
         <is>
-          <t>400, connection error</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F163" s="4" t="n"/>
@@ -5211,27 +5223,27 @@
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
         <is>
-          <t>TC-1107</t>
+          <t>TC-931</t>
         </is>
       </c>
       <c r="B164" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C164" s="4" t="inlineStr">
         <is>
-          <t>Provision — invalid database name</t>
+          <t>OS_GROUP_DELETED audit log</t>
         </is>
       </c>
       <c r="D164" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
         </is>
       </c>
       <c r="E164" s="4" t="inlineStr">
         <is>
-          <t>422, invalid identifier</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F164" s="4" t="n"/>
@@ -5240,60 +5252,48 @@
       <c r="I164" s="4" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="4" t="inlineStr">
-        <is>
-          <t>TC-1108</t>
-        </is>
-      </c>
-      <c r="B165" s="4" t="inlineStr">
-        <is>
-          <t>12.11 Database Provisioning</t>
-        </is>
-      </c>
-      <c r="C165" s="4" t="inlineStr">
-        <is>
-          <t>Status — connected</t>
-        </is>
-      </c>
-      <c r="D165" s="4" t="inlineStr">
-        <is>
-          <t>GET /setup/database/status with admin token</t>
-        </is>
-      </c>
-      <c r="E165" s="4" t="inlineStr">
-        <is>
-          <t>200, connected: true, migration info</t>
-        </is>
-      </c>
-      <c r="F165" s="4" t="n"/>
-      <c r="G165" s="4" t="n"/>
-      <c r="H165" s="4" t="n"/>
-      <c r="I165" s="4" t="n"/>
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>§12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="n"/>
+      <c r="D165" s="3" t="n"/>
+      <c r="E165" s="3" t="n"/>
+      <c r="F165" s="3" t="n"/>
+      <c r="G165" s="3" t="n"/>
+      <c r="H165" s="3" t="n"/>
+      <c r="I165" s="3" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
         <is>
-          <t>TC-1109</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B166" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C166" s="4" t="inlineStr">
         <is>
-          <t>Status — requires auth</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D166" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status without token</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E166" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F166" s="4" t="n"/>
@@ -5304,27 +5304,27 @@
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
         <is>
-          <t>TC-1110</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C167" s="4" t="inlineStr">
         <is>
-          <t>Status — requires admin</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>GET /setup/database/status with processor token</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E167" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F167" s="4" t="n"/>
@@ -5335,27 +5335,27 @@
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
         <is>
-          <t>TC-1111</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B168" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C168" s="4" t="inlineStr">
         <is>
-          <t>Settings update — success</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D168" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with valid partial update</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E168" s="4" t="inlineStr">
         <is>
-          <t>200, {"status": "updated", ...}</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F168" s="4" t="n"/>
@@ -5366,27 +5366,27 @@
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
         <is>
-          <t>TC-1112</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C169" s="4" t="inlineStr">
         <is>
-          <t>Settings update — bad connection</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with unreachable host</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E169" s="4" t="inlineStr">
         <is>
-          <t>400, connection test failed</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F169" s="4" t="n"/>
@@ -5397,27 +5397,27 @@
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
         <is>
-          <t>TC-1113</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B170" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C170" s="4" t="inlineStr">
         <is>
-          <t>Settings update — empty body</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D170" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with {}</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>422, at least one field required</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F170" s="4" t="n"/>
@@ -5428,27 +5428,27 @@
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
         <is>
-          <t>TC-1114</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C171" s="4" t="inlineStr">
         <is>
-          <t>Settings update — requires admin</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>PUT /setup/database/settings with processor token</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E171" s="4" t="inlineStr">
         <is>
-          <t>403</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F171" s="4" t="n"/>
@@ -5459,27 +5459,27 @@
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>TC-1115</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — test-connection</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E172" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F172" s="4" t="n"/>
@@ -5490,27 +5490,27 @@
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
         <is>
-          <t>TC-1116</t>
+          <t>TC-1008</t>
         </is>
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C173" s="4" t="inlineStr">
         <is>
-          <t>Auth after setup — provision</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D173" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision without token (after admin exists)</t>
+          <t>POST /auth/token with the admin credentials from step 2</t>
         </is>
       </c>
       <c r="E173" s="4" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F173" s="4" t="n"/>
@@ -5521,27 +5521,27 @@
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>TC-1117</t>
+          <t>TC-1009</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
         <is>
-          <t>12.11 Database Provisioning</t>
+          <t>12.10 First-Run Setup</t>
         </is>
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Password redaction</t>
+          <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision and check response</t>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
       <c r="E174" s="4" t="inlineStr">
         <is>
-          <t>No password in response body</t>
+          <t>Audit entry with actor</t>
         </is>
       </c>
       <c r="F174" s="4" t="n"/>
@@ -5550,40 +5550,28 @@
       <c r="I174" s="4" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="4" t="inlineStr">
-        <is>
-          <t>TC-1118</t>
-        </is>
-      </c>
-      <c r="B175" s="4" t="inlineStr">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>§12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C175" s="4" t="inlineStr">
-        <is>
-          <t>Re-provision blocked</t>
-        </is>
-      </c>
-      <c r="D175" s="4" t="inlineStr">
-        <is>
-          <t>POST /setup/database/provision after successful provisioning (no force)</t>
-        </is>
-      </c>
-      <c r="E175" s="4" t="inlineStr">
-        <is>
-          <t>409, already provisioned</t>
-        </is>
-      </c>
-      <c r="F175" s="4" t="n"/>
-      <c r="G175" s="4" t="n"/>
-      <c r="H175" s="4" t="n"/>
-      <c r="I175" s="4" t="n"/>
+      <c r="C175" s="3" t="n"/>
+      <c r="D175" s="3" t="n"/>
+      <c r="E175" s="3" t="n"/>
+      <c r="F175" s="3" t="n"/>
+      <c r="G175" s="3" t="n"/>
+      <c r="H175" s="3" t="n"/>
+      <c r="I175" s="3" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>TC-1119</t>
+          <t>TC-1101</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -5593,17 +5581,17 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision (admin)</t>
+          <t>Test connection — success</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
       <c r="E176" s="4" t="inlineStr">
         <is>
-          <t>200, returns database, user, migrations_applied</t>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
       <c r="F176" s="4" t="n"/>
@@ -5614,7 +5602,7 @@
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
         <is>
-          <t>TC-1120</t>
+          <t>TC-1102</t>
         </is>
       </c>
       <c r="B177" s="4" t="inlineStr">
@@ -5624,17 +5612,17 @@
       </c>
       <c r="C177" s="4" t="inlineStr">
         <is>
-          <t>Force rejected unauthenticated</t>
+          <t>Test connection — bad host</t>
         </is>
       </c>
       <c r="D177" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+          <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
       <c r="E177" s="4" t="inlineStr">
         <is>
-          <t>403, force requires admin</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F177" s="4" t="n"/>
@@ -5645,7 +5633,7 @@
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>TC-1121</t>
+          <t>TC-1103</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -5655,17 +5643,17 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Test connection — SSRF host</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>422, invalid host</t>
         </is>
       </c>
       <c r="F178" s="4" t="n"/>
@@ -5676,7 +5664,7 @@
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
         <is>
-          <t>TC-1122</t>
+          <t>TC-1104</t>
         </is>
       </c>
       <c r="B179" s="4" t="inlineStr">
@@ -5686,17 +5674,17 @@
       </c>
       <c r="C179" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Test connection — port out of range</t>
         </is>
       </c>
       <c r="D179" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
       <c r="E179" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F179" s="4" t="n"/>
@@ -5707,7 +5695,7 @@
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
         <is>
-          <t>TC-1123</t>
+          <t>TC-1105</t>
         </is>
       </c>
       <c r="B180" s="4" t="inlineStr">
@@ -5717,17 +5705,17 @@
       </c>
       <c r="C180" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — provision state unknown</t>
+          <t>Provision — success</t>
         </is>
       </c>
       <c r="D180" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+          <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
       <c r="E180" s="4" t="inlineStr">
         <is>
-          <t>503, cannot determine provisioning state</t>
+          <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
       <c r="F180" s="4" t="n"/>
@@ -5738,7 +5726,7 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>TC-1124</t>
+          <t>TC-1106</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
@@ -5748,17 +5736,17 @@
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>Force bypasses state check</t>
+          <t>Provision — bad admin credentials</t>
         </is>
       </c>
       <c r="D181" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+          <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
       <c r="E181" s="4" t="inlineStr">
         <is>
-          <t>Proceeds to provisioning (no 503 from state check)</t>
+          <t>400, connection error</t>
         </is>
       </c>
       <c r="F181" s="4" t="n"/>
@@ -5769,7 +5757,7 @@
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>TC-1125</t>
+          <t>TC-1107</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
@@ -5779,17 +5767,17 @@
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>Unmigrated DB treated as initial setup</t>
+          <t>Provision — invalid database name</t>
         </is>
       </c>
       <c r="D182" s="4" t="inlineStr">
         <is>
-          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
       <c r="E182" s="4" t="inlineStr">
         <is>
-          <t>200, request allowed (not 503)</t>
+          <t>422, invalid identifier</t>
         </is>
       </c>
       <c r="F182" s="4" t="n"/>
@@ -5800,7 +5788,7 @@
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>TC-1126</t>
+          <t>TC-1108</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
@@ -5810,17 +5798,17 @@
       </c>
       <c r="C183" s="4" t="inlineStr">
         <is>
-          <t>Fresh install — DB/role missing</t>
+          <t>Status — connected</t>
         </is>
       </c>
       <c r="D183" s="4" t="inlineStr">
         <is>
-          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+          <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
       <c r="E183" s="4" t="inlineStr">
         <is>
-          <t>200, provisioning proceeds (not 503)</t>
+          <t>200, connected: true, migration info</t>
         </is>
       </c>
       <c r="F183" s="4" t="n"/>
@@ -5831,7 +5819,7 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>TC-1127</t>
+          <t>TC-1109</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -5841,17 +5829,17 @@
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — OperationalError on reachable DB</t>
+          <t>Status — requires auth</t>
         </is>
       </c>
       <c r="D184" s="4" t="inlineStr">
         <is>
-          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status without token</t>
         </is>
       </c>
       <c r="E184" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>401</t>
         </is>
       </c>
       <c r="F184" s="4" t="n"/>
@@ -5862,7 +5850,7 @@
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>TC-1128</t>
+          <t>TC-1110</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
@@ -5872,17 +5860,17 @@
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — unexpected error</t>
+          <t>Status — requires admin</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
         <is>
-          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+          <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
       <c r="E185" s="4" t="inlineStr">
         <is>
-          <t>503, does NOT grant unauthenticated access</t>
+          <t>403</t>
         </is>
       </c>
       <c r="F185" s="4" t="n"/>
@@ -5893,7 +5881,7 @@
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>TC-1129</t>
+          <t>TC-1111</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
@@ -5903,17 +5891,17 @@
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>Provision — migration failure</t>
+          <t>Settings update — success</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+          <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
       <c r="E186" s="4" t="inlineStr">
         <is>
-          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+          <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
       <c r="F186" s="4" t="n"/>
@@ -5924,7 +5912,7 @@
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>TC-1130</t>
+          <t>TC-1112</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
@@ -5934,17 +5922,17 @@
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>Provision — .env write failure</t>
+          <t>Settings update — bad connection</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+          <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
       <c r="E187" s="4" t="inlineStr">
         <is>
-          <t>500, "failed to persist" message; engine not swapped</t>
+          <t>400, connection test failed</t>
         </is>
       </c>
       <c r="F187" s="4" t="n"/>
@@ -5955,7 +5943,7 @@
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>TC-1131</t>
+          <t>TC-1113</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
@@ -5965,17 +5953,17 @@
       </c>
       <c r="C188" s="4" t="inlineStr">
         <is>
-          <t>Provision — engine reinit failure</t>
+          <t>Settings update — empty body</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+          <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
       <c r="E188" s="4" t="inlineStr">
         <is>
-          <t>500, "engine could not be switched" message; .env already written</t>
+          <t>422, at least one field required</t>
         </is>
       </c>
       <c r="F188" s="4" t="n"/>
@@ -5983,14 +5971,572 @@
       <c r="H188" s="4" t="n"/>
       <c r="I188" s="4" t="n"/>
     </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>TC-1114</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>Settings update — requires admin</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>PUT /setup/database/settings with processor token</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="F189" s="4" t="n"/>
+      <c r="G189" s="4" t="n"/>
+      <c r="H189" s="4" t="n"/>
+      <c r="I189" s="4" t="n"/>
+    </row>
     <row r="190">
-      <c r="A190" s="5" t="inlineStr">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>TC-1115</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>Auth after setup — test-connection</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E190" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F190" s="4" t="n"/>
+      <c r="G190" s="4" t="n"/>
+      <c r="H190" s="4" t="n"/>
+      <c r="I190" s="4" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="4" t="inlineStr">
+        <is>
+          <t>TC-1116</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>Auth after setup — provision</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E191" s="4" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F191" s="4" t="n"/>
+      <c r="G191" s="4" t="n"/>
+      <c r="H191" s="4" t="n"/>
+      <c r="I191" s="4" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>TC-1117</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr">
+        <is>
+          <t>Password redaction</t>
+        </is>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision and check response</t>
+        </is>
+      </c>
+      <c r="E192" s="4" t="inlineStr">
+        <is>
+          <t>No password in response body</t>
+        </is>
+      </c>
+      <c r="F192" s="4" t="n"/>
+      <c r="G192" s="4" t="n"/>
+      <c r="H192" s="4" t="n"/>
+      <c r="I192" s="4" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>TC-1118</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr">
+        <is>
+          <t>Re-provision blocked</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+        </is>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>409, already provisioned</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="n"/>
+      <c r="G193" s="4" t="n"/>
+      <c r="H193" s="4" t="n"/>
+      <c r="I193" s="4" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="4" t="inlineStr">
+        <is>
+          <t>TC-1119</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C194" s="4" t="inlineStr">
+        <is>
+          <t>Force re-provision (admin)</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
+        </is>
+      </c>
+      <c r="E194" s="4" t="inlineStr">
+        <is>
+          <t>200, returns database, user, migrations_applied</t>
+        </is>
+      </c>
+      <c r="F194" s="4" t="n"/>
+      <c r="G194" s="4" t="n"/>
+      <c r="H194" s="4" t="n"/>
+      <c r="I194" s="4" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="4" t="inlineStr">
+        <is>
+          <t>TC-1120</t>
+        </is>
+      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C195" s="4" t="inlineStr">
+        <is>
+          <t>Force rejected unauthenticated</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="inlineStr">
+        <is>
+          <t>403, force requires admin</t>
+        </is>
+      </c>
+      <c r="F195" s="4" t="n"/>
+      <c r="G195" s="4" t="n"/>
+      <c r="H195" s="4" t="n"/>
+      <c r="I195" s="4" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>TC-1121</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, no JWT</t>
+        </is>
+      </c>
+      <c r="D196" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E196" s="4" t="inlineStr">
+        <is>
+          <t>503, database unavailable message</t>
+        </is>
+      </c>
+      <c r="F196" s="4" t="n"/>
+      <c r="G196" s="4" t="n"/>
+      <c r="H196" s="4" t="n"/>
+      <c r="I196" s="4" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="4" t="inlineStr">
+        <is>
+          <t>TC-1122</t>
+        </is>
+      </c>
+      <c r="B197" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C197" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
+        </is>
+      </c>
+      <c r="D197" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+        </is>
+      </c>
+      <c r="E197" s="4" t="inlineStr">
+        <is>
+          <t>Request proceeds (not blocked by 503)</t>
+        </is>
+      </c>
+      <c r="F197" s="4" t="n"/>
+      <c r="G197" s="4" t="n"/>
+      <c r="H197" s="4" t="n"/>
+      <c r="I197" s="4" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>TC-1123</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — provision state unknown</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="inlineStr">
+        <is>
+          <t>503, cannot determine provisioning state</t>
+        </is>
+      </c>
+      <c r="F198" s="4" t="n"/>
+      <c r="G198" s="4" t="n"/>
+      <c r="H198" s="4" t="n"/>
+      <c r="I198" s="4" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>TC-1124</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>Force bypasses state check</t>
+        </is>
+      </c>
+      <c r="D199" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+        </is>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="n"/>
+      <c r="G199" s="4" t="n"/>
+      <c r="H199" s="4" t="n"/>
+      <c r="I199" s="4" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>TC-1125</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>Unmigrated DB treated as initial setup</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E200" s="4" t="inlineStr">
+        <is>
+          <t>200, request allowed (not 503)</t>
+        </is>
+      </c>
+      <c r="F200" s="4" t="n"/>
+      <c r="G200" s="4" t="n"/>
+      <c r="H200" s="4" t="n"/>
+      <c r="I200" s="4" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>TC-1126</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>Fresh install — DB/role missing</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+        </is>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>200, provisioning proceeds (not 503)</t>
+        </is>
+      </c>
+      <c r="F201" s="4" t="n"/>
+      <c r="G201" s="4" t="n"/>
+      <c r="H201" s="4" t="n"/>
+      <c r="I201" s="4" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="4" t="inlineStr">
+        <is>
+          <t>TC-1127</t>
+        </is>
+      </c>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C202" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — OperationalError on reachable DB</t>
+        </is>
+      </c>
+      <c r="D202" s="4" t="inlineStr">
+        <is>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E202" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F202" s="4" t="n"/>
+      <c r="G202" s="4" t="n"/>
+      <c r="H202" s="4" t="n"/>
+      <c r="I202" s="4" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>TC-1128</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — unexpected error</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="n"/>
+      <c r="G203" s="4" t="n"/>
+      <c r="H203" s="4" t="n"/>
+      <c r="I203" s="4" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="4" t="inlineStr">
+        <is>
+          <t>TC-1129</t>
+        </is>
+      </c>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C204" s="4" t="inlineStr">
+        <is>
+          <t>Provision — migration failure</t>
+        </is>
+      </c>
+      <c r="D204" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+        </is>
+      </c>
+      <c r="E204" s="4" t="inlineStr">
+        <is>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+        </is>
+      </c>
+      <c r="F204" s="4" t="n"/>
+      <c r="G204" s="4" t="n"/>
+      <c r="H204" s="4" t="n"/>
+      <c r="I204" s="4" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="4" t="inlineStr">
+        <is>
+          <t>TC-1130</t>
+        </is>
+      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C205" s="4" t="inlineStr">
+        <is>
+          <t>Provision — .env write failure</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+        </is>
+      </c>
+      <c r="E205" s="4" t="inlineStr">
+        <is>
+          <t>500, "failed to persist" message; engine not swapped</t>
+        </is>
+      </c>
+      <c r="F205" s="4" t="n"/>
+      <c r="G205" s="4" t="n"/>
+      <c r="H205" s="4" t="n"/>
+      <c r="I205" s="4" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>TC-1131</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C206" s="4" t="inlineStr">
+        <is>
+          <t>Provision — engine reinit failure</t>
+        </is>
+      </c>
+      <c r="D206" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+        </is>
+      </c>
+      <c r="E206" s="4" t="inlineStr">
+        <is>
+          <t>500, "engine could not be switched" message; .env already written</t>
+        </is>
+      </c>
+      <c r="F206" s="4" t="n"/>
+      <c r="G206" s="4" t="n"/>
+      <c r="H206" s="4" t="n"/>
+      <c r="I206" s="4" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B190" s="5" t="n">
-        <v>173</v>
+      <c r="B208" s="5" t="n">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>